<commit_message>
save figures and add cosine similarity on manuscrit notebook
</commit_message>
<xml_diff>
--- a/modules/09_downstream_analysis/tables/Tables_S1.xlsx
+++ b/modules/09_downstream_analysis/tables/Tables_S1.xlsx
@@ -272,7 +272,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FEDC88"/>
+        <fgColor rgb="00FEE28F"/>
       </patternFill>
     </fill>
     <fill>
@@ -372,11 +372,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00CBE982"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor rgb="00E24731"/>
       </patternFill>
     </fill>
@@ -392,27 +387,32 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
+        <fgColor rgb="00EC5C3B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FCAA5F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DCF08F"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00036E3A"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DB382B"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
         <fgColor rgb="00EA5739"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00FCAA5F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DCF08F"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00036E3A"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="00DB382B"/>
       </patternFill>
     </fill>
     <fill>
@@ -499,190 +499,190 @@
     <xf numFmtId="0" fontId="4" fillId="35" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="68" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="66" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="54" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="69" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="64" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="70" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="65" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="71" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="75" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="72" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="76" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="73" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="58" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="50" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="60" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="67" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="28" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="24" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="37" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="20" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="40" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="29" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="44" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="54" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="45" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="70" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="30" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="64" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="71" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="31" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="46" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="55" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="62" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="65" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="72" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="75" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="11" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="32" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="47" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="56" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="63" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="57" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="13" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="12" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="48" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="66" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="73" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="76" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="33" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="43" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="41" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="17" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="18" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="19" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="34" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="39" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="4" fillId="74" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="38" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="51" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="36" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="21" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="58" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="25" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="49" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="22" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="59" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="50" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="42" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="60" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="68" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -1141,22 +1141,22 @@
       </c>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="4" t="n">
-        <v>0.2200268121914505</v>
+        <v>0.2200267937910924</v>
       </c>
       <c r="G2" s="4" t="n">
-        <v>0.1683015741702871</v>
+        <v>0.168301558884163</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>21.49409664080809</v>
+        <v>21.49409854059367</v>
       </c>
       <c r="I2" s="6" t="n">
-        <v>50.62513334069335</v>
+        <v>50.62513122853903</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>0.3514189918854048</v>
+        <v>0.3514189889291304</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>0.533214074334017</v>
+        <v>0.5332140313892965</v>
       </c>
       <c r="L2" s="7" t="inlineStr"/>
       <c r="M2" s="7" t="inlineStr"/>
@@ -1183,31 +1183,31 @@
       </c>
       <c r="E3" s="3" t="inlineStr"/>
       <c r="F3" s="4" t="n">
-        <v>1.051838517653308</v>
+        <v>1.05183415673438</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>0.8957753078364548</v>
+        <v>0.8906536601543372</v>
       </c>
       <c r="H3" s="4" t="n">
-        <v>0.8795100304219089</v>
+        <v>0.8807593317495764</v>
       </c>
       <c r="I3" s="4" t="n">
-        <v>1.080372210799027</v>
+        <v>1.080372181515371</v>
       </c>
       <c r="J3" s="4" t="n">
-        <v>1.02415904295585</v>
+        <v>1.022551281624978</v>
       </c>
       <c r="K3" s="4" t="n">
-        <v>1.267417743551106</v>
+        <v>1.299474222037198</v>
       </c>
       <c r="L3" s="8" t="n">
-        <v>2.811744301364591</v>
+        <v>2.811417438156464</v>
       </c>
       <c r="M3" s="4" t="n">
-        <v>6.219247745526937</v>
+        <v>6.219245810877839</v>
       </c>
       <c r="N3" s="9" t="n">
-        <v>3.58838770914496</v>
+        <v>3.588387431206568</v>
       </c>
     </row>
     <row r="4">
@@ -1231,31 +1231,31 @@
       </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="4" t="n">
-        <v>1.425651312693434</v>
+        <v>1.413721555365447</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>1.332976512086869</v>
+        <v>1.332976559261508</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>1.20685245770083</v>
+        <v>1.195678297235432</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>1.429316385274336</v>
+        <v>1.4293163814537</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>1.235234164296606</v>
+        <v>1.23665343997475</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>1.720404041190537</v>
+        <v>1.720403969033206</v>
       </c>
       <c r="L4" s="4" t="n">
-        <v>2.40187860170066</v>
+        <v>2.401878716598962</v>
       </c>
       <c r="M4" s="4" t="n">
-        <v>6.459821010721651</v>
+        <v>6.4598212557446</v>
       </c>
       <c r="N4" s="10" t="n">
-        <v>47.99949029989904</v>
+        <v>47.99950129068093</v>
       </c>
     </row>
     <row r="5">
@@ -1279,28 +1279,28 @@
       </c>
       <c r="E5" s="3" t="inlineStr"/>
       <c r="F5" s="11" t="n">
-        <v>35.71234304943492</v>
+        <v>35.71235845306735</v>
       </c>
       <c r="G5" s="12" t="n">
-        <v>130.1734249728129</v>
+        <v>130.1734408128576</v>
       </c>
       <c r="H5" s="13" t="n">
-        <v>31.18709507809289</v>
+        <v>31.18709815702108</v>
       </c>
       <c r="I5" s="14" t="n">
-        <v>51.46898066660339</v>
+        <v>51.46895724144699</v>
       </c>
       <c r="J5" s="15" t="n">
-        <v>76.02216445297887</v>
+        <v>76.02217639965397</v>
       </c>
       <c r="K5" s="16" t="n">
-        <v>28.9776644869193</v>
+        <v>28.9777072725128</v>
       </c>
       <c r="L5" s="17" t="n">
-        <v>85.39011138140592</v>
+        <v>85.39010890009284</v>
       </c>
       <c r="M5" s="18" t="n">
-        <v>272.8999297769984</v>
+        <v>272.8999798562783</v>
       </c>
       <c r="N5" s="7" t="inlineStr"/>
     </row>
@@ -1325,28 +1325,28 @@
       </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="19" t="n">
-        <v>37.88172427922759</v>
+        <v>37.86031593532573</v>
       </c>
       <c r="G6" s="20" t="n">
-        <v>41.73573981555229</v>
-      </c>
-      <c r="H6" s="21" t="n">
-        <v>24.23650750033931</v>
-      </c>
-      <c r="I6" s="22" t="n">
-        <v>55.16642999467154</v>
-      </c>
-      <c r="J6" s="23" t="n">
-        <v>12.00949609272832</v>
-      </c>
-      <c r="K6" s="20" t="n">
-        <v>53.21315344178439</v>
-      </c>
-      <c r="L6" s="14" t="n">
-        <v>65.24464755067758</v>
-      </c>
-      <c r="M6" s="24" t="n">
-        <v>311.7147344639482</v>
+        <v>41.73574956653894</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>22.85187759638281</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>50.66199715177527</v>
+      </c>
+      <c r="J6" s="21" t="n">
+        <v>11.83744697179398</v>
+      </c>
+      <c r="K6" s="19" t="n">
+        <v>53.4987475117704</v>
+      </c>
+      <c r="L6" s="22" t="n">
+        <v>68.83863193837416</v>
+      </c>
+      <c r="M6" s="23" t="n">
+        <v>311.7147899973531</v>
       </c>
       <c r="N6" s="7" t="inlineStr"/>
     </row>
@@ -1370,26 +1370,26 @@
         </is>
       </c>
       <c r="E7" s="3" t="inlineStr"/>
-      <c r="F7" s="25" t="n">
-        <v>62.03304557221185</v>
-      </c>
-      <c r="G7" s="26" t="n">
-        <v>148.4668401717332</v>
-      </c>
-      <c r="H7" s="27" t="n">
-        <v>76.84423106314108</v>
-      </c>
-      <c r="I7" s="28" t="n">
-        <v>57.63238422840502</v>
-      </c>
-      <c r="J7" s="28" t="n">
-        <v>59.99444455613283</v>
-      </c>
-      <c r="K7" s="29" t="n">
-        <v>65.23163328692711</v>
-      </c>
-      <c r="L7" s="30" t="n">
-        <v>98.46650978006322</v>
+      <c r="F7" s="24" t="n">
+        <v>62.03303306107324</v>
+      </c>
+      <c r="G7" s="25" t="n">
+        <v>148.4668819502482</v>
+      </c>
+      <c r="H7" s="26" t="n">
+        <v>76.84421513821283</v>
+      </c>
+      <c r="I7" s="27" t="n">
+        <v>57.63237238929146</v>
+      </c>
+      <c r="J7" s="27" t="n">
+        <v>59.99443765415912</v>
+      </c>
+      <c r="K7" s="28" t="n">
+        <v>65.23161820866173</v>
+      </c>
+      <c r="L7" s="29" t="n">
+        <v>102.164311049296</v>
       </c>
       <c r="M7" s="7" t="inlineStr"/>
       <c r="N7" s="7" t="inlineStr"/>
@@ -1414,29 +1414,29 @@
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
-      <c r="F8" s="31" t="n">
-        <v>74.48467560241735</v>
-      </c>
-      <c r="G8" s="32" t="n">
-        <v>104.3940763572625</v>
-      </c>
-      <c r="H8" s="29" t="n">
-        <v>61.64035170992094</v>
+      <c r="F8" s="30" t="n">
+        <v>74.48466787970074</v>
+      </c>
+      <c r="G8" s="31" t="n">
+        <v>104.3940646207261</v>
+      </c>
+      <c r="H8" s="28" t="n">
+        <v>61.64034062213479</v>
       </c>
       <c r="I8" s="22" t="n">
-        <v>56.50489513299858</v>
-      </c>
-      <c r="J8" s="28" t="n">
-        <v>60.38248360366835</v>
-      </c>
-      <c r="K8" s="33" t="n">
-        <v>158.861229182315</v>
-      </c>
-      <c r="L8" s="34" t="n">
-        <v>171.8155200993839</v>
-      </c>
-      <c r="M8" s="29" t="n">
-        <v>209.7127874518602</v>
+        <v>56.50489506820175</v>
+      </c>
+      <c r="J8" s="27" t="n">
+        <v>60.38248497218612</v>
+      </c>
+      <c r="K8" s="32" t="n">
+        <v>158.8612179029319</v>
+      </c>
+      <c r="L8" s="33" t="n">
+        <v>171.8154465425989</v>
+      </c>
+      <c r="M8" s="28" t="n">
+        <v>209.7127836498971</v>
       </c>
       <c r="N8" s="7" t="inlineStr"/>
     </row>
@@ -1460,29 +1460,29 @@
         </is>
       </c>
       <c r="E9" s="3" t="inlineStr"/>
-      <c r="F9" s="35" t="n">
-        <v>237.0753353744764</v>
-      </c>
-      <c r="G9" s="36" t="n">
-        <v>227.4793165285805</v>
-      </c>
-      <c r="H9" s="37" t="n">
-        <v>233.9202898948836</v>
-      </c>
-      <c r="I9" s="38" t="n">
-        <v>206.5055794725461</v>
-      </c>
-      <c r="J9" s="39" t="n">
-        <v>297.5863010402848</v>
-      </c>
-      <c r="K9" s="40" t="n">
-        <v>276.828169750968</v>
-      </c>
-      <c r="L9" s="41" t="n">
-        <v>346.4295918708406</v>
-      </c>
-      <c r="M9" s="42" t="n">
-        <v>490.1378531983791</v>
+      <c r="F9" s="34" t="n">
+        <v>237.6827043466365</v>
+      </c>
+      <c r="G9" s="35" t="n">
+        <v>227.4793643886287</v>
+      </c>
+      <c r="H9" s="36" t="n">
+        <v>244.3758103183272</v>
+      </c>
+      <c r="I9" s="37" t="n">
+        <v>206.5056236502744</v>
+      </c>
+      <c r="J9" s="38" t="n">
+        <v>297.5781294634129</v>
+      </c>
+      <c r="K9" s="39" t="n">
+        <v>276.7663932738027</v>
+      </c>
+      <c r="L9" s="40" t="n">
+        <v>346.775470664047</v>
+      </c>
+      <c r="M9" s="41" t="n">
+        <v>490.137680054161</v>
       </c>
       <c r="N9" s="7" t="inlineStr"/>
     </row>
@@ -1506,32 +1506,32 @@
         </is>
       </c>
       <c r="E10" s="3" t="inlineStr"/>
-      <c r="F10" s="43" t="n">
-        <v>310.4890244650134</v>
-      </c>
-      <c r="G10" s="44" t="n">
-        <v>282.4733106203015</v>
-      </c>
-      <c r="H10" s="45" t="n">
-        <v>296.9220758950935</v>
-      </c>
-      <c r="I10" s="46" t="n">
-        <v>345.9169598604632</v>
-      </c>
-      <c r="J10" s="39" t="n">
-        <v>297.2128348789014</v>
-      </c>
-      <c r="K10" s="47" t="n">
-        <v>350.4309801218</v>
-      </c>
-      <c r="L10" s="48" t="n">
-        <v>464.5553257452278</v>
-      </c>
-      <c r="M10" s="28" t="n">
-        <v>241.7648536355197</v>
-      </c>
-      <c r="N10" s="49" t="n">
-        <v>316.3883016273167</v>
+      <c r="F10" s="42" t="n">
+        <v>310.4890218543081</v>
+      </c>
+      <c r="G10" s="43" t="n">
+        <v>282.4733035127171</v>
+      </c>
+      <c r="H10" s="44" t="n">
+        <v>296.922059686005</v>
+      </c>
+      <c r="I10" s="45" t="n">
+        <v>345.9169535365147</v>
+      </c>
+      <c r="J10" s="38" t="n">
+        <v>297.2128219253141</v>
+      </c>
+      <c r="K10" s="46" t="n">
+        <v>350.4309829414079</v>
+      </c>
+      <c r="L10" s="47" t="n">
+        <v>464.5553396628754</v>
+      </c>
+      <c r="M10" s="27" t="n">
+        <v>241.7648493408797</v>
+      </c>
+      <c r="N10" s="48" t="n">
+        <v>316.3883046601443</v>
       </c>
     </row>
     <row r="11">
@@ -1554,29 +1554,29 @@
         </is>
       </c>
       <c r="E11" s="3" t="inlineStr"/>
-      <c r="F11" s="50" t="n">
-        <v>318.6722923790113</v>
-      </c>
-      <c r="G11" s="49" t="n">
-        <v>495.0537810063217</v>
-      </c>
-      <c r="H11" s="51" t="n">
-        <v>331.4252090251458</v>
-      </c>
-      <c r="I11" s="48" t="n">
-        <v>370.374064031964</v>
-      </c>
-      <c r="J11" s="47" t="n">
-        <v>276.937568151968</v>
-      </c>
-      <c r="K11" s="52" t="n">
-        <v>386.1147073127026</v>
-      </c>
-      <c r="L11" s="53" t="n">
-        <v>576.2241598812321</v>
-      </c>
-      <c r="M11" s="54" t="n">
-        <v>1009.363766601537</v>
+      <c r="F11" s="49" t="n">
+        <v>318.3728346101513</v>
+      </c>
+      <c r="G11" s="48" t="n">
+        <v>495.0537324884929</v>
+      </c>
+      <c r="H11" s="50" t="n">
+        <v>331.4251957416804</v>
+      </c>
+      <c r="I11" s="47" t="n">
+        <v>370.3740342676523</v>
+      </c>
+      <c r="J11" s="46" t="n">
+        <v>276.9375767057196</v>
+      </c>
+      <c r="K11" s="38" t="n">
+        <v>377.8087360001696</v>
+      </c>
+      <c r="L11" s="51" t="n">
+        <v>576.2240991676478</v>
+      </c>
+      <c r="M11" s="52" t="n">
+        <v>1009.363833665608</v>
       </c>
       <c r="N11" s="7" t="inlineStr"/>
     </row>
@@ -1600,29 +1600,29 @@
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
-      <c r="F12" s="49" t="n">
-        <v>434.7568508465185</v>
-      </c>
-      <c r="G12" s="55" t="n">
-        <v>415.7683206295404</v>
-      </c>
-      <c r="H12" s="49" t="n">
-        <v>596.2549006374861</v>
-      </c>
-      <c r="I12" s="49" t="n">
-        <v>466.5253634397314</v>
-      </c>
-      <c r="J12" s="49" t="n">
-        <v>487.093637963118</v>
-      </c>
-      <c r="K12" s="49" t="n">
-        <v>616.8041483210507</v>
-      </c>
-      <c r="L12" s="49" t="n">
-        <v>584.9744151204068</v>
-      </c>
-      <c r="M12" s="49" t="n">
-        <v>1990.519104303546</v>
+      <c r="F12" s="48" t="n">
+        <v>434.7568920648509</v>
+      </c>
+      <c r="G12" s="53" t="n">
+        <v>415.7682831961437</v>
+      </c>
+      <c r="H12" s="48" t="n">
+        <v>596.2549665104681</v>
+      </c>
+      <c r="I12" s="48" t="n">
+        <v>466.5254378637795</v>
+      </c>
+      <c r="J12" s="48" t="n">
+        <v>487.093711510302</v>
+      </c>
+      <c r="K12" s="48" t="n">
+        <v>616.804240763021</v>
+      </c>
+      <c r="L12" s="48" t="n">
+        <v>584.9744821647076</v>
+      </c>
+      <c r="M12" s="48" t="n">
+        <v>1990.519699104975</v>
       </c>
       <c r="N12" s="7" t="inlineStr"/>
     </row>
@@ -1645,7 +1645,7 @@
           <t>Ashwagandha</t>
         </is>
       </c>
-      <c r="E13" s="56" t="inlineStr">
+      <c r="E13" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1679,7 +1679,7 @@
           <t>Comfrey</t>
         </is>
       </c>
-      <c r="E14" s="56" t="inlineStr">
+      <c r="E14" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -1698,7 +1698,7 @@
       <c r="A15" s="1" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="57" t="inlineStr">
+      <c r="B15" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1715,38 +1715,38 @@
       </c>
       <c r="E15" s="3" t="inlineStr"/>
       <c r="F15" s="4" t="n">
-        <v>0.1468538272398052</v>
+        <v>0.1494062749307615</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>0.0934087201709468</v>
+        <v>0.09340872882290333</v>
       </c>
       <c r="H15" s="4" t="n">
-        <v>0.1106234118539095</v>
+        <v>0.1110955191768163</v>
       </c>
       <c r="I15" s="4" t="n">
-        <v>0.1382365061323252</v>
+        <v>0.1463385779388922</v>
       </c>
       <c r="J15" s="4" t="n">
-        <v>0.1640352336235081</v>
+        <v>0.1715617894458027</v>
       </c>
       <c r="K15" s="4" t="n">
-        <v>0.2432665111857178</v>
+        <v>0.2490949610585927</v>
       </c>
       <c r="L15" s="4" t="n">
-        <v>0.3192853884572839</v>
+        <v>0.3199742946301236</v>
       </c>
       <c r="M15" s="4" t="n">
-        <v>0.1681854793119361</v>
+        <v>0.1681855220610241</v>
       </c>
       <c r="N15" s="4" t="n">
-        <v>0.398975097386051</v>
+        <v>0.3989751141119008</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1" t="n">
         <v>14</v>
       </c>
-      <c r="B16" s="57" t="inlineStr">
+      <c r="B16" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1763,38 +1763,38 @@
       </c>
       <c r="E16" s="3" t="inlineStr"/>
       <c r="F16" s="4" t="n">
-        <v>0.2151251031866624</v>
+        <v>0.2151251689107818</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>0.2406468497017566</v>
+        <v>0.2212206533050023</v>
       </c>
       <c r="H16" s="4" t="n">
-        <v>0.1354477123091527</v>
+        <v>0.1416719960998781</v>
       </c>
       <c r="I16" s="4" t="n">
-        <v>0.1374218619096253</v>
+        <v>0.137421867714111</v>
       </c>
       <c r="J16" s="4" t="n">
-        <v>0.1577086391753423</v>
+        <v>0.1577086820514984</v>
       </c>
       <c r="K16" s="4" t="n">
-        <v>0.4143626132783133</v>
+        <v>0.4129121449577219</v>
       </c>
       <c r="L16" s="4" t="n">
-        <v>0.7157987241776755</v>
+        <v>0.6686645096509554</v>
       </c>
       <c r="M16" s="4" t="n">
-        <v>1.306645928488177</v>
-      </c>
-      <c r="N16" s="58" t="n">
-        <v>19.03091332091493</v>
+        <v>1.306646247999758</v>
+      </c>
+      <c r="N16" s="56" t="n">
+        <v>19.03091474249145</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="57" t="inlineStr">
+      <c r="B17" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1811,38 +1811,38 @@
       </c>
       <c r="E17" s="3" t="inlineStr"/>
       <c r="F17" s="4" t="n">
-        <v>0.3003790190907911</v>
+        <v>0.3003265962032083</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>0.367312313160205</v>
+        <v>0.3673124588870912</v>
       </c>
       <c r="H17" s="4" t="n">
-        <v>0.7285845046149273</v>
+        <v>0.6693344016572341</v>
       </c>
       <c r="I17" s="4" t="n">
-        <v>0.1741922719445424</v>
+        <v>0.1737029220931279</v>
       </c>
       <c r="J17" s="4" t="n">
-        <v>0.737144075177724</v>
+        <v>0.7371441636949816</v>
       </c>
       <c r="K17" s="4" t="n">
-        <v>0.2335106909879373</v>
+        <v>0.2335107066274851</v>
       </c>
       <c r="L17" s="4" t="n">
-        <v>0.2637956516153416</v>
+        <v>0.2637956976939187</v>
       </c>
       <c r="M17" s="4" t="n">
-        <v>1.774397280713867</v>
-      </c>
-      <c r="N17" s="59" t="n">
-        <v>17.96187877227807</v>
+        <v>1.774397604074023</v>
+      </c>
+      <c r="N17" s="57" t="n">
+        <v>17.96188096926021</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="57" t="inlineStr">
+      <c r="B18" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1859,25 +1859,25 @@
       </c>
       <c r="E18" s="3" t="inlineStr"/>
       <c r="F18" s="4" t="n">
-        <v>0.5795355352876147</v>
+        <v>0.5795356064886886</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>0.5249639542818257</v>
+        <v>0.5249639912226558</v>
       </c>
       <c r="H18" s="20" t="n">
-        <v>49.52943901589399</v>
+        <v>49.52944166887266</v>
       </c>
       <c r="I18" s="8" t="n">
-        <v>3.235101657432746</v>
+        <v>3.235101812688842</v>
       </c>
       <c r="J18" s="9" t="n">
-        <v>4.271582519355218</v>
+        <v>4.271582474623628</v>
       </c>
       <c r="K18" s="4" t="n">
-        <v>1.974135612319155</v>
+        <v>1.974135810656127</v>
       </c>
       <c r="L18" s="4" t="n">
-        <v>1.262856939207609</v>
+        <v>1.262857041533183</v>
       </c>
       <c r="M18" s="7" t="inlineStr"/>
       <c r="N18" s="7" t="inlineStr"/>
@@ -1886,7 +1886,7 @@
       <c r="A19" s="1" t="n">
         <v>17</v>
       </c>
-      <c r="B19" s="57" t="inlineStr">
+      <c r="B19" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1903,38 +1903,38 @@
       </c>
       <c r="E19" s="3" t="inlineStr"/>
       <c r="F19" s="4" t="n">
-        <v>0.7778291080584153</v>
+        <v>0.7779473128631068</v>
       </c>
       <c r="G19" s="4" t="n">
-        <v>0.4339572762327132</v>
+        <v>0.4339574423033091</v>
       </c>
       <c r="H19" s="4" t="n">
-        <v>0.6631212151071655</v>
+        <v>0.6628700843747118</v>
       </c>
       <c r="I19" s="4" t="n">
-        <v>0.9953145949572739</v>
+        <v>0.9953148572838877</v>
       </c>
       <c r="J19" s="4" t="n">
-        <v>0.7519673865278121</v>
+        <v>0.7519676213084633</v>
       </c>
       <c r="K19" s="4" t="n">
-        <v>1.030992222286627</v>
+        <v>1.045356430886328</v>
       </c>
       <c r="L19" s="4" t="n">
-        <v>1.211539469154502</v>
+        <v>1.211539825997619</v>
       </c>
       <c r="M19" s="4" t="n">
-        <v>0.8644525658182671</v>
-      </c>
-      <c r="N19" s="60" t="n">
-        <v>4.303508499527231</v>
+        <v>0.8644528010725691</v>
+      </c>
+      <c r="N19" s="58" t="n">
+        <v>4.303509429801921</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="1" t="n">
         <v>18</v>
       </c>
-      <c r="B20" s="57" t="inlineStr">
+      <c r="B20" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1951,28 +1951,28 @@
       </c>
       <c r="E20" s="3" t="inlineStr"/>
       <c r="F20" s="4" t="n">
-        <v>1.129727103347552</v>
-      </c>
-      <c r="G20" s="61" t="n">
-        <v>7.837105921533632</v>
+        <v>1.129727140612866</v>
+      </c>
+      <c r="G20" s="59" t="n">
+        <v>7.837106251987495</v>
       </c>
       <c r="H20" s="4" t="n">
-        <v>0.5782891251584605</v>
-      </c>
-      <c r="I20" s="62" t="n">
-        <v>10.08907296603625</v>
-      </c>
-      <c r="J20" s="62" t="n">
-        <v>10.86996573019171</v>
-      </c>
-      <c r="K20" s="62" t="n">
-        <v>14.4875366559857</v>
-      </c>
-      <c r="L20" s="21" t="n">
-        <v>23.88685288361911</v>
-      </c>
-      <c r="M20" s="23" t="n">
-        <v>48.90912675001721</v>
+        <v>0.578289137765289</v>
+      </c>
+      <c r="I20" s="60" t="n">
+        <v>10.08907327823569</v>
+      </c>
+      <c r="J20" s="60" t="n">
+        <v>10.8699663182732</v>
+      </c>
+      <c r="K20" s="60" t="n">
+        <v>14.48753744252084</v>
+      </c>
+      <c r="L20" s="61" t="n">
+        <v>23.88685518503102</v>
+      </c>
+      <c r="M20" s="21" t="n">
+        <v>48.90912528215949</v>
       </c>
       <c r="N20" s="7" t="inlineStr"/>
     </row>
@@ -1980,7 +1980,7 @@
       <c r="A21" s="1" t="n">
         <v>19</v>
       </c>
-      <c r="B21" s="57" t="inlineStr">
+      <c r="B21" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -1997,38 +1997,38 @@
       </c>
       <c r="E21" s="3" t="inlineStr"/>
       <c r="F21" s="4" t="n">
-        <v>1.266989923775282</v>
+        <v>1.258466919431326</v>
       </c>
       <c r="G21" s="4" t="n">
-        <v>1.206916544924074</v>
+        <v>1.206916789698066</v>
       </c>
       <c r="H21" s="4" t="n">
-        <v>1.099481667516685</v>
+        <v>1.078010823518248</v>
       </c>
       <c r="I21" s="4" t="n">
-        <v>1.46997638810762</v>
+        <v>1.475136018112048</v>
       </c>
       <c r="J21" s="4" t="n">
-        <v>1.24511057575406</v>
+        <v>1.193474705550352</v>
       </c>
       <c r="K21" s="4" t="n">
-        <v>1.280486161927565</v>
+        <v>1.270794479132227</v>
       </c>
       <c r="L21" s="4" t="n">
-        <v>1.518176824864863</v>
+        <v>1.518177122055019</v>
       </c>
       <c r="M21" s="4" t="n">
-        <v>2.231753611821154</v>
+        <v>2.231753955200286</v>
       </c>
       <c r="N21" s="13" t="n">
-        <v>17.57982372597885</v>
+        <v>17.57982372002923</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="1" t="n">
         <v>20</v>
       </c>
-      <c r="B22" s="57" t="inlineStr">
+      <c r="B22" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2045,28 +2045,28 @@
       </c>
       <c r="E22" s="3" t="inlineStr"/>
       <c r="F22" s="8" t="n">
-        <v>2.146412104680529</v>
-      </c>
-      <c r="G22" s="63" t="n">
-        <v>36.06473280771086</v>
+        <v>2.146412309298834</v>
+      </c>
+      <c r="G22" s="62" t="n">
+        <v>36.06473518460834</v>
       </c>
       <c r="H22" s="4" t="n">
-        <v>0.320673556900922</v>
+        <v>0.3206735527400296</v>
       </c>
       <c r="I22" s="8" t="n">
-        <v>2.430636562442972</v>
+        <v>2.430637019459291</v>
       </c>
       <c r="J22" s="8" t="n">
-        <v>2.932304840706212</v>
-      </c>
-      <c r="K22" s="60" t="n">
-        <v>7.658459375887043</v>
-      </c>
-      <c r="L22" s="61" t="n">
-        <v>9.471526124796533</v>
+        <v>2.932305130760063</v>
+      </c>
+      <c r="K22" s="58" t="n">
+        <v>7.658459726246471</v>
+      </c>
+      <c r="L22" s="59" t="n">
+        <v>9.471526884075256</v>
       </c>
       <c r="M22" s="5" t="n">
-        <v>73.56921589904888</v>
+        <v>73.56921120872579</v>
       </c>
       <c r="N22" s="7" t="inlineStr"/>
     </row>
@@ -2074,7 +2074,7 @@
       <c r="A23" s="1" t="n">
         <v>21</v>
       </c>
-      <c r="B23" s="57" t="inlineStr">
+      <c r="B23" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2091,28 +2091,28 @@
       </c>
       <c r="E23" s="3" t="inlineStr"/>
       <c r="F23" s="8" t="n">
-        <v>2.37018119980501</v>
+        <v>2.370181631147835</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>4.349556003868839</v>
+        <v>4.349557760835272</v>
       </c>
       <c r="H23" s="8" t="n">
-        <v>3.47785085157784</v>
+        <v>3.477851493154576</v>
       </c>
       <c r="I23" s="8" t="n">
-        <v>3.500424270200518</v>
+        <v>3.599921728177987</v>
       </c>
       <c r="J23" s="8" t="n">
-        <v>3.04886129453005</v>
+        <v>3.048861956091458</v>
       </c>
       <c r="K23" s="4" t="n">
-        <v>0.4658053558775666</v>
+        <v>0.4658053949252655</v>
       </c>
       <c r="L23" s="8" t="n">
-        <v>4.005395503059732</v>
+        <v>4.005396440767435</v>
       </c>
       <c r="M23" s="8" t="n">
-        <v>15.45286760196678</v>
+        <v>15.45287066177693</v>
       </c>
       <c r="N23" s="7" t="inlineStr"/>
     </row>
@@ -2120,7 +2120,7 @@
       <c r="A24" s="1" t="n">
         <v>22</v>
       </c>
-      <c r="B24" s="57" t="inlineStr">
+      <c r="B24" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2137,38 +2137,38 @@
       </c>
       <c r="E24" s="3" t="inlineStr"/>
       <c r="F24" s="8" t="n">
-        <v>2.424561616772727</v>
+        <v>2.423725390755514</v>
       </c>
       <c r="G24" s="8" t="n">
-        <v>2.83351354948021</v>
+        <v>2.991541148024853</v>
       </c>
       <c r="H24" s="4" t="n">
-        <v>1.954495626038337</v>
+        <v>1.954495926922945</v>
       </c>
       <c r="I24" s="8" t="n">
-        <v>2.533150946781009</v>
+        <v>2.533151258694037</v>
       </c>
       <c r="J24" s="4" t="n">
-        <v>1.890847518465716</v>
+        <v>1.890847877089461</v>
       </c>
       <c r="K24" s="4" t="n">
-        <v>2.171493045333556</v>
+        <v>2.171493253786045</v>
       </c>
       <c r="L24" s="8" t="n">
-        <v>3.608552218648354</v>
+        <v>3.637911105372036</v>
       </c>
       <c r="M24" s="4" t="n">
-        <v>6.138627363937863</v>
+        <v>6.13862780526486</v>
       </c>
       <c r="N24" s="5" t="n">
-        <v>12.25009138874985</v>
+        <v>12.25009151710469</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="1" t="n">
         <v>23</v>
       </c>
-      <c r="B25" s="57" t="inlineStr">
+      <c r="B25" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2185,25 +2185,25 @@
       </c>
       <c r="E25" s="3" t="inlineStr"/>
       <c r="F25" s="8" t="n">
-        <v>3.487564186604458</v>
+        <v>3.514922032167785</v>
       </c>
       <c r="G25" s="4" t="n">
-        <v>0.9223707148497929</v>
+        <v>0.922371067347648</v>
       </c>
       <c r="H25" s="8" t="n">
-        <v>4.741305466861181</v>
+        <v>4.741306352333545</v>
       </c>
       <c r="I25" s="9" t="n">
-        <v>4.799779195406176</v>
+        <v>5.026143797009471</v>
       </c>
       <c r="J25" s="9" t="n">
-        <v>4.217275484661075</v>
+        <v>4.21727587073029</v>
       </c>
       <c r="K25" s="9" t="n">
-        <v>5.550321320483859</v>
+        <v>5.550321794943253</v>
       </c>
       <c r="L25" s="9" t="n">
-        <v>6.580273498314067</v>
+        <v>6.580274819477131</v>
       </c>
       <c r="M25" s="7" t="inlineStr"/>
       <c r="N25" s="7" t="inlineStr"/>
@@ -2212,7 +2212,7 @@
       <c r="A26" s="1" t="n">
         <v>24</v>
       </c>
-      <c r="B26" s="57" t="inlineStr">
+      <c r="B26" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2229,28 +2229,28 @@
       </c>
       <c r="E26" s="3" t="inlineStr"/>
       <c r="F26" s="9" t="n">
-        <v>3.642194351000399</v>
+        <v>3.642194480393004</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>5.598730974593309</v>
+        <v>5.598731348998613</v>
       </c>
       <c r="H26" s="8" t="n">
-        <v>2.564820442217028</v>
-      </c>
-      <c r="I26" s="61" t="n">
-        <v>9.200655296718038</v>
-      </c>
-      <c r="J26" s="61" t="n">
-        <v>9.014558982833213</v>
+        <v>2.564820582634759</v>
+      </c>
+      <c r="I26" s="59" t="n">
+        <v>9.20065616898963</v>
+      </c>
+      <c r="J26" s="59" t="n">
+        <v>9.014561295479483</v>
       </c>
       <c r="K26" s="9" t="n">
-        <v>5.571376862101698</v>
-      </c>
-      <c r="L26" s="61" t="n">
-        <v>9.586539026333128</v>
+        <v>5.571377988363365</v>
+      </c>
+      <c r="L26" s="59" t="n">
+        <v>9.586540252845744</v>
       </c>
       <c r="M26" s="5" t="n">
-        <v>72.20972295040747</v>
+        <v>72.2097081419936</v>
       </c>
       <c r="N26" s="7" t="inlineStr"/>
     </row>
@@ -2258,7 +2258,7 @@
       <c r="A27" s="1" t="n">
         <v>25</v>
       </c>
-      <c r="B27" s="57" t="inlineStr">
+      <c r="B27" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2275,25 +2275,25 @@
       </c>
       <c r="E27" s="3" t="inlineStr"/>
       <c r="F27" s="9" t="n">
-        <v>4.295503615677756</v>
+        <v>4.295503919617376</v>
       </c>
       <c r="G27" s="16" t="n">
-        <v>21.78380879198932</v>
+        <v>21.78380955616702</v>
       </c>
       <c r="H27" s="5" t="n">
-        <v>22.84800461770662</v>
-      </c>
-      <c r="I27" s="62" t="n">
-        <v>10.59470972835189</v>
-      </c>
-      <c r="J27" s="23" t="n">
-        <v>13.08241439484794</v>
+        <v>22.84800714380074</v>
+      </c>
+      <c r="I27" s="60" t="n">
+        <v>10.59470857619369</v>
+      </c>
+      <c r="J27" s="21" t="n">
+        <v>13.08241539316306</v>
       </c>
       <c r="K27" s="9" t="n">
-        <v>6.050062074562187</v>
-      </c>
-      <c r="L27" s="64" t="n">
-        <v>54.85280226792884</v>
+        <v>6.050062442592708</v>
+      </c>
+      <c r="L27" s="63" t="n">
+        <v>54.85280175828015</v>
       </c>
       <c r="M27" s="7" t="inlineStr"/>
       <c r="N27" s="7" t="inlineStr"/>
@@ -2302,7 +2302,7 @@
       <c r="A28" s="1" t="n">
         <v>26</v>
       </c>
-      <c r="B28" s="57" t="inlineStr">
+      <c r="B28" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2319,28 +2319,28 @@
       </c>
       <c r="E28" s="3" t="inlineStr"/>
       <c r="F28" s="9" t="n">
-        <v>4.604809945176954</v>
+        <v>4.604810143609433</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>4.656588346486593</v>
+        <v>4.656588638643187</v>
       </c>
       <c r="H28" s="9" t="n">
-        <v>5.658508718725424</v>
-      </c>
-      <c r="I28" s="60" t="n">
-        <v>6.33917268163415</v>
-      </c>
-      <c r="J28" s="61" t="n">
-        <v>7.832691125002409</v>
+        <v>5.658509039603424</v>
+      </c>
+      <c r="I28" s="58" t="n">
+        <v>6.339173022018104</v>
+      </c>
+      <c r="J28" s="59" t="n">
+        <v>7.832691669917573</v>
       </c>
       <c r="K28" s="9" t="n">
-        <v>6.615240715615404</v>
+        <v>6.615241127604849</v>
       </c>
       <c r="L28" s="4" t="n">
-        <v>0.3145699407577457</v>
-      </c>
-      <c r="M28" s="21" t="n">
-        <v>85.23000933340359</v>
+        <v>0.3145699027410392</v>
+      </c>
+      <c r="M28" s="61" t="n">
+        <v>85.22998943447546</v>
       </c>
       <c r="N28" s="7" t="inlineStr"/>
     </row>
@@ -2348,7 +2348,7 @@
       <c r="A29" s="1" t="n">
         <v>27</v>
       </c>
-      <c r="B29" s="57" t="inlineStr">
+      <c r="B29" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2364,39 +2364,39 @@
         </is>
       </c>
       <c r="E29" s="3" t="inlineStr"/>
-      <c r="F29" s="60" t="n">
-        <v>5.942697902702214</v>
-      </c>
-      <c r="G29" s="60" t="n">
-        <v>7.670634967853651</v>
+      <c r="F29" s="58" t="n">
+        <v>5.93194464786618</v>
+      </c>
+      <c r="G29" s="58" t="n">
+        <v>7.670634986988253</v>
       </c>
       <c r="H29" s="9" t="n">
-        <v>6.345454302199139</v>
-      </c>
-      <c r="I29" s="61" t="n">
-        <v>8.582155097892379</v>
+        <v>6.072056873954425</v>
+      </c>
+      <c r="I29" s="59" t="n">
+        <v>8.58215530922147</v>
       </c>
       <c r="J29" s="9" t="n">
-        <v>5.843122725249362</v>
+        <v>5.843122684699095</v>
       </c>
       <c r="K29" s="9" t="n">
-        <v>7.113053443138808</v>
+        <v>7.113053458169043</v>
       </c>
       <c r="L29" s="9" t="n">
-        <v>5.206332361296322</v>
+        <v>5.206332415431604</v>
       </c>
       <c r="M29" s="4" t="n">
-        <v>6.709276321728835</v>
-      </c>
-      <c r="N29" s="65" t="n">
-        <v>37.30871656903624</v>
+        <v>6.709276221188672</v>
+      </c>
+      <c r="N29" s="64" t="n">
+        <v>37.30871491413358</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
         <v>28</v>
       </c>
-      <c r="B30" s="57" t="inlineStr">
+      <c r="B30" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2412,39 +2412,39 @@
         </is>
       </c>
       <c r="E30" s="3" t="inlineStr"/>
-      <c r="F30" s="60" t="n">
-        <v>6.006088522846914</v>
-      </c>
-      <c r="G30" s="60" t="n">
-        <v>5.967185767313487</v>
+      <c r="F30" s="58" t="n">
+        <v>6.015730767697116</v>
+      </c>
+      <c r="G30" s="58" t="n">
+        <v>5.967185724444796</v>
       </c>
       <c r="H30" s="9" t="n">
-        <v>6.913851443167318</v>
+        <v>6.902194873190855</v>
       </c>
       <c r="I30" s="9" t="n">
-        <v>4.675402806508985</v>
-      </c>
-      <c r="J30" s="60" t="n">
-        <v>6.004273166394251</v>
+        <v>4.850061637845833</v>
+      </c>
+      <c r="J30" s="58" t="n">
+        <v>6.004273267735075</v>
       </c>
       <c r="K30" s="9" t="n">
-        <v>7.16715926931523</v>
-      </c>
-      <c r="L30" s="60" t="n">
-        <v>9.170995138970747</v>
-      </c>
-      <c r="M30" s="61" t="n">
-        <v>35.97485972588532</v>
-      </c>
-      <c r="N30" s="66" t="n">
-        <v>23.92294534189752</v>
+        <v>7.140663109758324</v>
+      </c>
+      <c r="L30" s="58" t="n">
+        <v>9.281575185138212</v>
+      </c>
+      <c r="M30" s="59" t="n">
+        <v>35.97486237511421</v>
+      </c>
+      <c r="N30" s="65" t="n">
+        <v>23.92294489268524</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="1" t="n">
         <v>29</v>
       </c>
-      <c r="B31" s="57" t="inlineStr">
+      <c r="B31" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2460,39 +2460,39 @@
         </is>
       </c>
       <c r="E31" s="3" t="inlineStr"/>
-      <c r="F31" s="60" t="n">
-        <v>6.15010807006975</v>
+      <c r="F31" s="58" t="n">
+        <v>6.185131717433828</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>5.152881737161683</v>
+        <v>5.152881707682763</v>
       </c>
       <c r="H31" s="9" t="n">
-        <v>6.888057141436342</v>
-      </c>
-      <c r="I31" s="60" t="n">
-        <v>6.573203430848161</v>
-      </c>
-      <c r="J31" s="9" t="n">
-        <v>5.232807457690641</v>
+        <v>6.888057071040582</v>
+      </c>
+      <c r="I31" s="58" t="n">
+        <v>6.573203415812539</v>
+      </c>
+      <c r="J31" s="58" t="n">
+        <v>5.948189440714222</v>
       </c>
       <c r="K31" s="9" t="n">
-        <v>6.61579578885522</v>
+        <v>6.615795789368277</v>
       </c>
       <c r="L31" s="9" t="n">
-        <v>5.469438601567644</v>
-      </c>
-      <c r="M31" s="23" t="n">
-        <v>48.79454939389416</v>
-      </c>
-      <c r="N31" s="67" t="n">
-        <v>30.61188958208811</v>
+        <v>5.469438617286984</v>
+      </c>
+      <c r="M31" s="21" t="n">
+        <v>48.79454793974083</v>
+      </c>
+      <c r="N31" s="66" t="n">
+        <v>30.61189046331645</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="1" t="n">
         <v>30</v>
       </c>
-      <c r="B32" s="57" t="inlineStr">
+      <c r="B32" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2508,26 +2508,26 @@
         </is>
       </c>
       <c r="E32" s="3" t="inlineStr"/>
-      <c r="F32" s="60" t="n">
-        <v>6.433576951679038</v>
-      </c>
-      <c r="G32" s="68" t="n">
-        <v>32.23285214267393</v>
+      <c r="F32" s="58" t="n">
+        <v>6.433577221314078</v>
+      </c>
+      <c r="G32" s="67" t="n">
+        <v>32.23285158126562</v>
       </c>
       <c r="H32" s="16" t="n">
-        <v>26.92365443774877</v>
-      </c>
-      <c r="I32" s="60" t="n">
-        <v>6.121914287985812</v>
-      </c>
-      <c r="J32" s="69" t="n">
-        <v>15.10841278087474</v>
+        <v>26.92365392666587</v>
+      </c>
+      <c r="I32" s="58" t="n">
+        <v>6.121914466574262</v>
+      </c>
+      <c r="J32" s="68" t="n">
+        <v>15.10841448077675</v>
       </c>
       <c r="K32" s="8" t="n">
-        <v>4.855696878452837</v>
+        <v>4.855697193178676</v>
       </c>
       <c r="L32" s="9" t="n">
-        <v>6.381346806742128</v>
+        <v>6.381347587923905</v>
       </c>
       <c r="M32" s="7" t="inlineStr"/>
       <c r="N32" s="7" t="inlineStr"/>
@@ -2536,7 +2536,7 @@
       <c r="A33" s="1" t="n">
         <v>31</v>
       </c>
-      <c r="B33" s="57" t="inlineStr">
+      <c r="B33" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2552,29 +2552,29 @@
         </is>
       </c>
       <c r="E33" s="3" t="inlineStr"/>
-      <c r="F33" s="60" t="n">
-        <v>6.917057631333098</v>
+      <c r="F33" s="58" t="n">
+        <v>6.91705839422842</v>
       </c>
       <c r="G33" s="22" t="n">
-        <v>58.11127877882176</v>
-      </c>
-      <c r="H33" s="62" t="n">
-        <v>12.92128985777142</v>
-      </c>
-      <c r="I33" s="70" t="n">
-        <v>84.2879893455481</v>
-      </c>
-      <c r="J33" s="60" t="n">
-        <v>6.372984998807604</v>
+        <v>58.11127717443146</v>
+      </c>
+      <c r="H33" s="60" t="n">
+        <v>12.92129028430582</v>
+      </c>
+      <c r="I33" s="69" t="n">
+        <v>84.28799518952249</v>
+      </c>
+      <c r="J33" s="58" t="n">
+        <v>6.372985132635971</v>
       </c>
       <c r="K33" s="5" t="n">
-        <v>22.38608316334722</v>
-      </c>
-      <c r="L33" s="23" t="n">
-        <v>14.66193696356166</v>
-      </c>
-      <c r="M33" s="71" t="n">
-        <v>94.71644872749849</v>
+        <v>22.38608370893749</v>
+      </c>
+      <c r="L33" s="21" t="n">
+        <v>14.66193798518666</v>
+      </c>
+      <c r="M33" s="70" t="n">
+        <v>94.71643184449606</v>
       </c>
       <c r="N33" s="7" t="inlineStr"/>
     </row>
@@ -2582,7 +2582,7 @@
       <c r="A34" s="1" t="n">
         <v>32</v>
       </c>
-      <c r="B34" s="57" t="inlineStr">
+      <c r="B34" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2598,29 +2598,29 @@
         </is>
       </c>
       <c r="E34" s="3" t="inlineStr"/>
-      <c r="F34" s="61" t="n">
-        <v>7.101371642299432</v>
-      </c>
-      <c r="G34" s="66" t="n">
-        <v>38.6628705698546</v>
-      </c>
-      <c r="H34" s="72" t="n">
-        <v>79.48659571885884</v>
+      <c r="F34" s="59" t="n">
+        <v>7.101372361025989</v>
+      </c>
+      <c r="G34" s="65" t="n">
+        <v>38.66286920330591</v>
+      </c>
+      <c r="H34" s="71" t="n">
+        <v>79.48647609325991</v>
       </c>
       <c r="I34" s="13" t="n">
-        <v>24.76472300746289</v>
-      </c>
-      <c r="J34" s="23" t="n">
-        <v>11.80364883411488</v>
+        <v>24.76472525359642</v>
+      </c>
+      <c r="J34" s="21" t="n">
+        <v>11.80364935335409</v>
       </c>
       <c r="K34" s="18" t="n">
-        <v>86.45811892954258</v>
+        <v>86.4581061319648</v>
       </c>
       <c r="L34" s="9" t="n">
-        <v>5.878378242427514</v>
+        <v>5.878378931833743</v>
       </c>
       <c r="M34" s="16" t="n">
-        <v>87.24874010181398</v>
+        <v>87.24872856325021</v>
       </c>
       <c r="N34" s="7" t="inlineStr"/>
     </row>
@@ -2628,7 +2628,7 @@
       <c r="A35" s="1" t="n">
         <v>33</v>
       </c>
-      <c r="B35" s="57" t="inlineStr">
+      <c r="B35" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2644,29 +2644,29 @@
         </is>
       </c>
       <c r="E35" s="3" t="inlineStr"/>
-      <c r="F35" s="61" t="n">
-        <v>7.380347272780479</v>
-      </c>
-      <c r="G35" s="71" t="n">
-        <v>24.32931243868719</v>
+      <c r="F35" s="59" t="n">
+        <v>7.380349236621822</v>
+      </c>
+      <c r="G35" s="70" t="n">
+        <v>24.32931252502762</v>
       </c>
       <c r="H35" s="9" t="n">
-        <v>6.055337854346797</v>
-      </c>
-      <c r="I35" s="60" t="n">
-        <v>6.444089566921691</v>
-      </c>
-      <c r="J35" s="60" t="n">
-        <v>7.587969421098878</v>
-      </c>
-      <c r="K35" s="61" t="n">
-        <v>10.8000709396939</v>
-      </c>
-      <c r="L35" s="61" t="n">
-        <v>9.778064430706403</v>
-      </c>
-      <c r="M35" s="73" t="n">
-        <v>68.93653432792377</v>
+        <v>6.06016836119571</v>
+      </c>
+      <c r="I35" s="58" t="n">
+        <v>6.444090329807256</v>
+      </c>
+      <c r="J35" s="58" t="n">
+        <v>7.587972196906483</v>
+      </c>
+      <c r="K35" s="59" t="n">
+        <v>10.8000721854289</v>
+      </c>
+      <c r="L35" s="59" t="n">
+        <v>9.778065780363331</v>
+      </c>
+      <c r="M35" s="72" t="n">
+        <v>68.93650441137201</v>
       </c>
       <c r="N35" s="7" t="inlineStr"/>
     </row>
@@ -2674,7 +2674,7 @@
       <c r="A36" s="1" t="n">
         <v>34</v>
       </c>
-      <c r="B36" s="57" t="inlineStr">
+      <c r="B36" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2690,29 +2690,29 @@
         </is>
       </c>
       <c r="E36" s="3" t="inlineStr"/>
-      <c r="F36" s="61" t="n">
-        <v>7.595789154107631</v>
-      </c>
-      <c r="G36" s="73" t="n">
-        <v>15.9090881567691</v>
-      </c>
-      <c r="H36" s="61" t="n">
-        <v>9.617036891818744</v>
-      </c>
-      <c r="I36" s="61" t="n">
-        <v>7.757529686826787</v>
-      </c>
-      <c r="J36" s="61" t="n">
-        <v>9.361240091040321</v>
+      <c r="F36" s="59" t="n">
+        <v>7.595790902668268</v>
+      </c>
+      <c r="G36" s="72" t="n">
+        <v>15.90908986977204</v>
+      </c>
+      <c r="H36" s="59" t="n">
+        <v>9.617037797156401</v>
+      </c>
+      <c r="I36" s="59" t="n">
+        <v>7.757531041739865</v>
+      </c>
+      <c r="J36" s="59" t="n">
+        <v>9.361240745158463</v>
       </c>
       <c r="K36" s="4" t="n">
-        <v>2.562548375099366</v>
-      </c>
-      <c r="L36" s="62" t="n">
-        <v>12.5455628868828</v>
-      </c>
-      <c r="M36" s="21" t="n">
-        <v>84.55647292449916</v>
+        <v>2.56254850233897</v>
+      </c>
+      <c r="L36" s="60" t="n">
+        <v>12.54556400143658</v>
+      </c>
+      <c r="M36" s="61" t="n">
+        <v>84.55646011321402</v>
       </c>
       <c r="N36" s="7" t="inlineStr"/>
     </row>
@@ -2720,7 +2720,7 @@
       <c r="A37" s="1" t="n">
         <v>35</v>
       </c>
-      <c r="B37" s="57" t="inlineStr">
+      <c r="B37" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2736,29 +2736,29 @@
         </is>
       </c>
       <c r="E37" s="3" t="inlineStr"/>
-      <c r="F37" s="61" t="n">
-        <v>7.731927763188256</v>
+      <c r="F37" s="59" t="n">
+        <v>7.731929327136231</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>5.085001577375618</v>
-      </c>
-      <c r="H37" s="62" t="n">
-        <v>12.68338427427843</v>
-      </c>
-      <c r="I37" s="61" t="n">
-        <v>8.166189713496253</v>
-      </c>
-      <c r="J37" s="23" t="n">
-        <v>11.66010593998979</v>
-      </c>
-      <c r="K37" s="60" t="n">
-        <v>9.145789548383142</v>
-      </c>
-      <c r="L37" s="61" t="n">
-        <v>9.505871675651925</v>
+        <v>5.085002469111175</v>
+      </c>
+      <c r="H37" s="60" t="n">
+        <v>12.68338482351086</v>
+      </c>
+      <c r="I37" s="59" t="n">
+        <v>8.166191115328886</v>
+      </c>
+      <c r="J37" s="21" t="n">
+        <v>11.66010915184447</v>
+      </c>
+      <c r="K37" s="58" t="n">
+        <v>9.145789919668147</v>
+      </c>
+      <c r="L37" s="59" t="n">
+        <v>9.505873017187954</v>
       </c>
       <c r="M37" s="9" t="n">
-        <v>22.7186727624756</v>
+        <v>22.71868351383771</v>
       </c>
       <c r="N37" s="7" t="inlineStr"/>
     </row>
@@ -2766,7 +2766,7 @@
       <c r="A38" s="1" t="n">
         <v>36</v>
       </c>
-      <c r="B38" s="57" t="inlineStr">
+      <c r="B38" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2782,29 +2782,29 @@
         </is>
       </c>
       <c r="E38" s="3" t="inlineStr"/>
-      <c r="F38" s="61" t="n">
-        <v>7.859945509025711</v>
-      </c>
-      <c r="G38" s="73" t="n">
-        <v>17.1136440370216</v>
-      </c>
-      <c r="H38" s="23" t="n">
-        <v>16.13727148842603</v>
+      <c r="F38" s="59" t="n">
+        <v>7.859945872927365</v>
+      </c>
+      <c r="G38" s="72" t="n">
+        <v>17.11364756712201</v>
+      </c>
+      <c r="H38" s="21" t="n">
+        <v>16.13727126235521</v>
       </c>
       <c r="I38" s="5" t="n">
-        <v>17.5959389169239</v>
-      </c>
-      <c r="J38" s="72" t="n">
-        <v>66.24501070709191</v>
-      </c>
-      <c r="K38" s="69" t="n">
-        <v>18.58666065895591</v>
+        <v>17.59593770240829</v>
+      </c>
+      <c r="J38" s="71" t="n">
+        <v>66.24500368908581</v>
+      </c>
+      <c r="K38" s="68" t="n">
+        <v>18.58666014351696</v>
       </c>
       <c r="L38" s="20" t="n">
-        <v>50.08388146558184</v>
-      </c>
-      <c r="M38" s="21" t="n">
-        <v>79.72065722841953</v>
+        <v>50.08388370366844</v>
+      </c>
+      <c r="M38" s="61" t="n">
+        <v>79.7206453002505</v>
       </c>
       <c r="N38" s="7" t="inlineStr"/>
     </row>
@@ -2812,7 +2812,7 @@
       <c r="A39" s="1" t="n">
         <v>37</v>
       </c>
-      <c r="B39" s="57" t="inlineStr">
+      <c r="B39" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2828,24 +2828,24 @@
         </is>
       </c>
       <c r="E39" s="3" t="inlineStr"/>
-      <c r="F39" s="61" t="n">
-        <v>8.060076316286537</v>
+      <c r="F39" s="59" t="n">
+        <v>8.06007663216846</v>
       </c>
       <c r="G39" s="11" t="n">
-        <v>39.88275620264745</v>
+        <v>39.88275908091259</v>
       </c>
       <c r="H39" s="9" t="n">
-        <v>5.265917627835405</v>
-      </c>
-      <c r="I39" s="27" t="n">
-        <v>59.50138930358614</v>
-      </c>
-      <c r="J39" s="58" t="n">
-        <v>30.23463478002084</v>
+        <v>5.265917822978576</v>
+      </c>
+      <c r="I39" s="26" t="n">
+        <v>59.50139834947755</v>
+      </c>
+      <c r="J39" s="56" t="n">
+        <v>30.23463510040747</v>
       </c>
       <c r="K39" s="7" t="inlineStr"/>
-      <c r="L39" s="64" t="n">
-        <v>53.14405353534353</v>
+      <c r="L39" s="63" t="n">
+        <v>53.14405092660811</v>
       </c>
       <c r="M39" s="7" t="inlineStr"/>
       <c r="N39" s="7" t="inlineStr"/>
@@ -2854,7 +2854,7 @@
       <c r="A40" s="1" t="n">
         <v>38</v>
       </c>
-      <c r="B40" s="57" t="inlineStr">
+      <c r="B40" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2870,26 +2870,26 @@
         </is>
       </c>
       <c r="E40" s="3" t="inlineStr"/>
-      <c r="F40" s="61" t="n">
-        <v>8.398473433785805</v>
-      </c>
-      <c r="G40" s="71" t="n">
-        <v>23.50603645660326</v>
-      </c>
-      <c r="H40" s="60" t="n">
-        <v>8.894458817986779</v>
-      </c>
-      <c r="I40" s="73" t="n">
-        <v>14.94218749328705</v>
+      <c r="F40" s="59" t="n">
+        <v>8.398473586197944</v>
+      </c>
+      <c r="G40" s="70" t="n">
+        <v>23.50603722868411</v>
+      </c>
+      <c r="H40" s="58" t="n">
+        <v>8.894459172186432</v>
+      </c>
+      <c r="I40" s="72" t="n">
+        <v>14.94218882764894</v>
       </c>
       <c r="J40" s="9" t="n">
-        <v>4.282078922374971</v>
-      </c>
-      <c r="K40" s="60" t="n">
-        <v>8.902303256709978</v>
-      </c>
-      <c r="L40" s="60" t="n">
-        <v>8.570424193805897</v>
+        <v>4.282079114238042</v>
+      </c>
+      <c r="K40" s="58" t="n">
+        <v>8.902293487245247</v>
+      </c>
+      <c r="L40" s="58" t="n">
+        <v>8.57042440253282</v>
       </c>
       <c r="M40" s="7" t="inlineStr"/>
       <c r="N40" s="7" t="inlineStr"/>
@@ -2898,7 +2898,7 @@
       <c r="A41" s="1" t="n">
         <v>39</v>
       </c>
-      <c r="B41" s="57" t="inlineStr">
+      <c r="B41" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2914,29 +2914,29 @@
         </is>
       </c>
       <c r="E41" s="3" t="inlineStr"/>
-      <c r="F41" s="62" t="n">
-        <v>9.168912594777735</v>
-      </c>
-      <c r="G41" s="21" t="n">
-        <v>21.32361814243069</v>
-      </c>
-      <c r="H41" s="62" t="n">
-        <v>13.47190078519511</v>
-      </c>
-      <c r="I41" s="60" t="n">
-        <v>7.033350391151814</v>
-      </c>
-      <c r="J41" s="59" t="n">
-        <v>26.90155960315153</v>
-      </c>
-      <c r="K41" s="59" t="n">
-        <v>35.11560137211764</v>
-      </c>
-      <c r="L41" s="61" t="n">
-        <v>9.893352796193563</v>
-      </c>
-      <c r="M41" s="71" t="n">
-        <v>96.02089093619549</v>
+      <c r="F41" s="60" t="n">
+        <v>9.168912930513272</v>
+      </c>
+      <c r="G41" s="61" t="n">
+        <v>21.32362079097204</v>
+      </c>
+      <c r="H41" s="60" t="n">
+        <v>13.47190103045879</v>
+      </c>
+      <c r="I41" s="58" t="n">
+        <v>7.033350716543417</v>
+      </c>
+      <c r="J41" s="57" t="n">
+        <v>26.90156039377276</v>
+      </c>
+      <c r="K41" s="57" t="n">
+        <v>35.1156017719338</v>
+      </c>
+      <c r="L41" s="59" t="n">
+        <v>9.89335320641327</v>
+      </c>
+      <c r="M41" s="70" t="n">
+        <v>96.0208989416916</v>
       </c>
       <c r="N41" s="7" t="inlineStr"/>
     </row>
@@ -2944,7 +2944,7 @@
       <c r="A42" s="1" t="n">
         <v>40</v>
       </c>
-      <c r="B42" s="57" t="inlineStr">
+      <c r="B42" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -2960,29 +2960,29 @@
         </is>
       </c>
       <c r="E42" s="3" t="inlineStr"/>
-      <c r="F42" s="23" t="n">
-        <v>10.85920949549691</v>
-      </c>
-      <c r="G42" s="64" t="n">
-        <v>44.89715518711973</v>
-      </c>
-      <c r="H42" s="23" t="n">
-        <v>15.87472872542365</v>
-      </c>
-      <c r="I42" s="61" t="n">
-        <v>8.17939069818476</v>
-      </c>
-      <c r="J42" s="59" t="n">
-        <v>27.03611983887601</v>
+      <c r="F42" s="21" t="n">
+        <v>10.85921043432263</v>
+      </c>
+      <c r="G42" s="63" t="n">
+        <v>44.8971537680096</v>
+      </c>
+      <c r="H42" s="21" t="n">
+        <v>15.87473135268238</v>
+      </c>
+      <c r="I42" s="59" t="n">
+        <v>8.179391401332197</v>
+      </c>
+      <c r="J42" s="57" t="n">
+        <v>27.03611926511357</v>
       </c>
       <c r="K42" s="5" t="n">
-        <v>23.89206918563721</v>
-      </c>
-      <c r="L42" s="69" t="n">
-        <v>17.05312312434172</v>
+        <v>23.89207181755537</v>
+      </c>
+      <c r="L42" s="68" t="n">
+        <v>17.05312469974536</v>
       </c>
       <c r="M42" s="5" t="n">
-        <v>73.95215512469306</v>
+        <v>73.95214285722425</v>
       </c>
       <c r="N42" s="7" t="inlineStr"/>
     </row>
@@ -2990,7 +2990,7 @@
       <c r="A43" s="1" t="n">
         <v>41</v>
       </c>
-      <c r="B43" s="57" t="inlineStr">
+      <c r="B43" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3006,29 +3006,29 @@
         </is>
       </c>
       <c r="E43" s="3" t="inlineStr"/>
-      <c r="F43" s="23" t="n">
-        <v>10.97271648181081</v>
-      </c>
-      <c r="G43" s="69" t="n">
-        <v>15.10639761493733</v>
-      </c>
-      <c r="H43" s="73" t="n">
-        <v>20.65458504932136</v>
-      </c>
-      <c r="I43" s="69" t="n">
-        <v>14.18470482534973</v>
-      </c>
-      <c r="J43" s="60" t="n">
-        <v>6.729973766778006</v>
-      </c>
-      <c r="K43" s="23" t="n">
-        <v>16.03966934291861</v>
-      </c>
-      <c r="L43" s="58" t="n">
-        <v>36.64670725875439</v>
+      <c r="F43" s="21" t="n">
+        <v>10.97271821077574</v>
+      </c>
+      <c r="G43" s="68" t="n">
+        <v>15.10639892097537</v>
+      </c>
+      <c r="H43" s="72" t="n">
+        <v>20.65458672789782</v>
+      </c>
+      <c r="I43" s="68" t="n">
+        <v>14.18470684880022</v>
+      </c>
+      <c r="J43" s="58" t="n">
+        <v>6.72997447274474</v>
+      </c>
+      <c r="K43" s="21" t="n">
+        <v>16.03967093745567</v>
+      </c>
+      <c r="L43" s="56" t="n">
+        <v>36.64670526490959</v>
       </c>
       <c r="M43" s="16" t="n">
-        <v>92.12543502835285</v>
+        <v>92.12541938647627</v>
       </c>
       <c r="N43" s="7" t="inlineStr"/>
     </row>
@@ -3036,7 +3036,7 @@
       <c r="A44" s="1" t="n">
         <v>42</v>
       </c>
-      <c r="B44" s="57" t="inlineStr">
+      <c r="B44" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3052,37 +3052,37 @@
         </is>
       </c>
       <c r="E44" s="3" t="inlineStr"/>
-      <c r="F44" s="23" t="n">
-        <v>11.49527550689362</v>
-      </c>
-      <c r="G44" s="68" t="n">
-        <v>31.29818743458445</v>
-      </c>
-      <c r="H44" s="23" t="n">
-        <v>14.3568958644397</v>
-      </c>
-      <c r="I44" s="74" t="n">
-        <v>82.31250133847325</v>
-      </c>
-      <c r="J44" s="61" t="n">
-        <v>8.946973101779781</v>
-      </c>
-      <c r="K44" s="69" t="n">
-        <v>19.48066113037857</v>
+      <c r="F44" s="21" t="n">
+        <v>11.49527688815847</v>
+      </c>
+      <c r="G44" s="67" t="n">
+        <v>31.29819012118673</v>
+      </c>
+      <c r="H44" s="21" t="n">
+        <v>14.35689632271524</v>
+      </c>
+      <c r="I44" s="73" t="n">
+        <v>82.31250703998933</v>
+      </c>
+      <c r="J44" s="59" t="n">
+        <v>8.946974038870103</v>
+      </c>
+      <c r="K44" s="68" t="n">
+        <v>19.48066217720787</v>
       </c>
       <c r="L44" s="13" t="n">
-        <v>32.02747403075329</v>
+        <v>32.02747430078354</v>
       </c>
       <c r="M44" s="7" t="inlineStr"/>
-      <c r="N44" s="42" t="n">
-        <v>79.01174647220347</v>
+      <c r="N44" s="41" t="n">
+        <v>79.0117370618236</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1" t="n">
         <v>43</v>
       </c>
-      <c r="B45" s="57" t="inlineStr">
+      <c r="B45" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3098,29 +3098,29 @@
         </is>
       </c>
       <c r="E45" s="3" t="inlineStr"/>
-      <c r="F45" s="23" t="n">
-        <v>11.58024687437167</v>
-      </c>
-      <c r="G45" s="24" t="n">
-        <v>78.36011227402511</v>
+      <c r="F45" s="21" t="n">
+        <v>11.58024679853928</v>
+      </c>
+      <c r="G45" s="23" t="n">
+        <v>78.3601184262979</v>
       </c>
       <c r="H45" s="20" t="n">
-        <v>50.87654516380695</v>
-      </c>
-      <c r="I45" s="23" t="n">
-        <v>12.51324562009724</v>
-      </c>
-      <c r="J45" s="58" t="n">
-        <v>29.38074375479206</v>
-      </c>
-      <c r="K45" s="23" t="n">
-        <v>14.95091622049864</v>
-      </c>
-      <c r="L45" s="60" t="n">
-        <v>9.21863270163597</v>
-      </c>
-      <c r="M45" s="73" t="n">
-        <v>64.85122397929506</v>
+        <v>50.87654613429437</v>
+      </c>
+      <c r="I45" s="21" t="n">
+        <v>12.51324610942929</v>
+      </c>
+      <c r="J45" s="56" t="n">
+        <v>29.38074556808369</v>
+      </c>
+      <c r="K45" s="21" t="n">
+        <v>14.95091658377486</v>
+      </c>
+      <c r="L45" s="58" t="n">
+        <v>9.218633118370471</v>
+      </c>
+      <c r="M45" s="72" t="n">
+        <v>64.85121275739648</v>
       </c>
       <c r="N45" s="7" t="inlineStr"/>
     </row>
@@ -3128,7 +3128,7 @@
       <c r="A46" s="1" t="n">
         <v>44</v>
       </c>
-      <c r="B46" s="57" t="inlineStr">
+      <c r="B46" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3144,39 +3144,39 @@
         </is>
       </c>
       <c r="E46" s="3" t="inlineStr"/>
-      <c r="F46" s="69" t="n">
-        <v>12.06111626598067</v>
-      </c>
-      <c r="G46" s="23" t="n">
-        <v>11.77944727496453</v>
-      </c>
-      <c r="H46" s="60" t="n">
-        <v>7.941203656395919</v>
-      </c>
-      <c r="I46" s="61" t="n">
-        <v>7.793141091311188</v>
+      <c r="F46" s="68" t="n">
+        <v>12.06111632627596</v>
+      </c>
+      <c r="G46" s="21" t="n">
+        <v>11.77944734682332</v>
+      </c>
+      <c r="H46" s="58" t="n">
+        <v>7.941203838412907</v>
+      </c>
+      <c r="I46" s="59" t="n">
+        <v>7.793141130270071</v>
       </c>
       <c r="J46" s="5" t="n">
-        <v>17.89417335419492</v>
-      </c>
-      <c r="K46" s="62" t="n">
-        <v>13.17890434174658</v>
-      </c>
-      <c r="L46" s="69" t="n">
-        <v>18.13335494592149</v>
-      </c>
-      <c r="M46" s="73" t="n">
-        <v>65.89784069669163</v>
+        <v>17.89417400697478</v>
+      </c>
+      <c r="K46" s="60" t="n">
+        <v>13.17890443493395</v>
+      </c>
+      <c r="L46" s="68" t="n">
+        <v>18.13335534608877</v>
+      </c>
+      <c r="M46" s="72" t="n">
+        <v>65.89783232977233</v>
       </c>
       <c r="N46" s="12" t="n">
-        <v>84.23447915743566</v>
+        <v>84.23447926179813</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="1" t="n">
         <v>45</v>
       </c>
-      <c r="B47" s="57" t="inlineStr">
+      <c r="B47" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3192,24 +3192,24 @@
         </is>
       </c>
       <c r="E47" s="3" t="inlineStr"/>
-      <c r="F47" s="69" t="n">
-        <v>12.40865596158634</v>
+      <c r="F47" s="68" t="n">
+        <v>12.40865666615371</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>4.423432341124871</v>
-      </c>
-      <c r="H47" s="59" t="n">
-        <v>34.21531468847881</v>
-      </c>
-      <c r="I47" s="23" t="n">
-        <v>12.68606219986056</v>
+        <v>4.423432470731356</v>
+      </c>
+      <c r="H47" s="57" t="n">
+        <v>34.21531513951029</v>
+      </c>
+      <c r="I47" s="21" t="n">
+        <v>12.68606289694443</v>
       </c>
       <c r="J47" s="7" t="inlineStr"/>
-      <c r="K47" s="59" t="n">
-        <v>35.11384225156309</v>
+      <c r="K47" s="57" t="n">
+        <v>35.11384851833296</v>
       </c>
       <c r="L47" s="5" t="n">
-        <v>22.6077432169574</v>
+        <v>22.60774387050618</v>
       </c>
       <c r="M47" s="7" t="inlineStr"/>
       <c r="N47" s="7" t="inlineStr"/>
@@ -3218,7 +3218,7 @@
       <c r="A48" s="1" t="n">
         <v>46</v>
       </c>
-      <c r="B48" s="57" t="inlineStr">
+      <c r="B48" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3234,29 +3234,29 @@
         </is>
       </c>
       <c r="E48" s="3" t="inlineStr"/>
-      <c r="F48" s="69" t="n">
-        <v>12.61888169457147</v>
-      </c>
-      <c r="G48" s="61" t="n">
-        <v>8.009075723992204</v>
+      <c r="F48" s="68" t="n">
+        <v>12.61888305821957</v>
+      </c>
+      <c r="G48" s="59" t="n">
+        <v>8.009076855118018</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>21.6365023846023</v>
-      </c>
-      <c r="I48" s="69" t="n">
-        <v>14.67935698425948</v>
-      </c>
-      <c r="J48" s="23" t="n">
-        <v>12.79755960996591</v>
-      </c>
-      <c r="K48" s="73" t="n">
-        <v>19.99648377706325</v>
-      </c>
-      <c r="L48" s="73" t="n">
-        <v>19.15444178225124</v>
-      </c>
-      <c r="M48" s="73" t="n">
-        <v>66.49097029378919</v>
+        <v>21.63650596891947</v>
+      </c>
+      <c r="I48" s="68" t="n">
+        <v>14.67935714441098</v>
+      </c>
+      <c r="J48" s="21" t="n">
+        <v>12.7975609057946</v>
+      </c>
+      <c r="K48" s="72" t="n">
+        <v>19.99648378729441</v>
+      </c>
+      <c r="L48" s="72" t="n">
+        <v>19.15444215481512</v>
+      </c>
+      <c r="M48" s="72" t="n">
+        <v>66.49095896500563</v>
       </c>
       <c r="N48" s="7" t="inlineStr"/>
     </row>
@@ -3264,7 +3264,7 @@
       <c r="A49" s="1" t="n">
         <v>47</v>
       </c>
-      <c r="B49" s="57" t="inlineStr">
+      <c r="B49" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3280,26 +3280,26 @@
         </is>
       </c>
       <c r="E49" s="3" t="inlineStr"/>
-      <c r="F49" s="69" t="n">
-        <v>13.5958100057878</v>
-      </c>
-      <c r="G49" s="64" t="n">
-        <v>45.00106271553872</v>
-      </c>
-      <c r="H49" s="73" t="n">
-        <v>19.26547821465306</v>
-      </c>
-      <c r="I49" s="62" t="n">
-        <v>9.451008599590773</v>
+      <c r="F49" s="68" t="n">
+        <v>13.59677732516242</v>
+      </c>
+      <c r="G49" s="63" t="n">
+        <v>45.00106423641317</v>
+      </c>
+      <c r="H49" s="72" t="n">
+        <v>19.26547845233046</v>
+      </c>
+      <c r="I49" s="60" t="n">
+        <v>9.45100970480255</v>
       </c>
       <c r="J49" s="5" t="n">
-        <v>18.92654772744642</v>
-      </c>
-      <c r="K49" s="62" t="n">
-        <v>12.82770067424437</v>
-      </c>
-      <c r="L49" s="23" t="n">
-        <v>14.73133001678277</v>
+        <v>18.92654818005123</v>
+      </c>
+      <c r="K49" s="60" t="n">
+        <v>12.82770076875769</v>
+      </c>
+      <c r="L49" s="21" t="n">
+        <v>14.8070782071109</v>
       </c>
       <c r="M49" s="7" t="inlineStr"/>
       <c r="N49" s="7" t="inlineStr"/>
@@ -3308,7 +3308,7 @@
       <c r="A50" s="1" t="n">
         <v>48</v>
       </c>
-      <c r="B50" s="57" t="inlineStr">
+      <c r="B50" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3324,24 +3324,24 @@
         </is>
       </c>
       <c r="E50" s="3" t="inlineStr"/>
-      <c r="F50" s="73" t="n">
-        <v>13.81911014861695</v>
+      <c r="F50" s="72" t="n">
+        <v>13.81911080378119</v>
       </c>
       <c r="G50" s="16" t="n">
-        <v>22.54401064138202</v>
-      </c>
-      <c r="H50" s="73" t="n">
-        <v>19.97991465863554</v>
+        <v>22.54401085159736</v>
+      </c>
+      <c r="H50" s="72" t="n">
+        <v>19.97991558586637</v>
       </c>
       <c r="I50" s="7" t="inlineStr"/>
-      <c r="J50" s="13" t="n">
-        <v>25.25262946595136</v>
-      </c>
-      <c r="K50" s="62" t="n">
-        <v>12.65167812680736</v>
+      <c r="J50" s="65" t="n">
+        <v>36.65573614926468</v>
+      </c>
+      <c r="K50" s="60" t="n">
+        <v>12.65167850349779</v>
       </c>
       <c r="L50" s="14" t="n">
-        <v>66.36995510617294</v>
+        <v>66.36995180406245</v>
       </c>
       <c r="M50" s="7" t="inlineStr"/>
       <c r="N50" s="7" t="inlineStr"/>
@@ -3350,7 +3350,7 @@
       <c r="A51" s="1" t="n">
         <v>49</v>
       </c>
-      <c r="B51" s="57" t="inlineStr">
+      <c r="B51" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3366,26 +3366,26 @@
         </is>
       </c>
       <c r="E51" s="3" t="inlineStr"/>
-      <c r="F51" s="73" t="n">
-        <v>14.36883146813753</v>
+      <c r="F51" s="72" t="n">
+        <v>14.3688329415992</v>
       </c>
       <c r="G51" s="13" t="n">
-        <v>26.88435451245678</v>
-      </c>
-      <c r="H51" s="21" t="n">
-        <v>24.10088619885392</v>
-      </c>
-      <c r="I51" s="75" t="n">
-        <v>32.53728939600548</v>
-      </c>
-      <c r="J51" s="62" t="n">
-        <v>10.70642639328073</v>
+        <v>26.88435617472693</v>
+      </c>
+      <c r="H51" s="61" t="n">
+        <v>24.10088898888355</v>
+      </c>
+      <c r="I51" s="74" t="n">
+        <v>32.53728733869172</v>
+      </c>
+      <c r="J51" s="60" t="n">
+        <v>10.70642775561487</v>
       </c>
       <c r="K51" s="5" t="n">
-        <v>22.87206830565486</v>
-      </c>
-      <c r="L51" s="24" t="n">
-        <v>92.24875955004089</v>
+        <v>22.87206941482775</v>
+      </c>
+      <c r="L51" s="23" t="n">
+        <v>92.24875075635849</v>
       </c>
       <c r="M51" s="7" t="inlineStr"/>
       <c r="N51" s="7" t="inlineStr"/>
@@ -3394,7 +3394,7 @@
       <c r="A52" s="1" t="n">
         <v>50</v>
       </c>
-      <c r="B52" s="57" t="inlineStr">
+      <c r="B52" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3411,25 +3411,25 @@
       </c>
       <c r="E52" s="3" t="inlineStr"/>
       <c r="F52" s="5" t="n">
-        <v>15.44356869505876</v>
+        <v>15.44382955899318</v>
       </c>
       <c r="G52" s="16" t="n">
-        <v>22.03658328727311</v>
-      </c>
-      <c r="H52" s="69" t="n">
-        <v>17.91496218989433</v>
-      </c>
-      <c r="I52" s="69" t="n">
-        <v>13.25749811465573</v>
-      </c>
-      <c r="J52" s="73" t="n">
-        <v>15.73914219374222</v>
-      </c>
-      <c r="K52" s="23" t="n">
-        <v>15.28337674200961</v>
-      </c>
-      <c r="L52" s="69" t="n">
-        <v>17.62429883740128</v>
+        <v>22.03658498875297</v>
+      </c>
+      <c r="H52" s="68" t="n">
+        <v>17.91496449587365</v>
+      </c>
+      <c r="I52" s="68" t="n">
+        <v>13.25749968480366</v>
+      </c>
+      <c r="J52" s="72" t="n">
+        <v>15.73919404158632</v>
+      </c>
+      <c r="K52" s="21" t="n">
+        <v>15.31033606182026</v>
+      </c>
+      <c r="L52" s="68" t="n">
+        <v>17.6243010335262</v>
       </c>
       <c r="M52" s="7" t="inlineStr"/>
       <c r="N52" s="7" t="inlineStr"/>
@@ -3438,7 +3438,7 @@
       <c r="A53" s="1" t="n">
         <v>51</v>
       </c>
-      <c r="B53" s="57" t="inlineStr">
+      <c r="B53" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3455,28 +3455,28 @@
       </c>
       <c r="E53" s="3" t="inlineStr"/>
       <c r="F53" s="5" t="n">
-        <v>16.51408837679644</v>
-      </c>
-      <c r="G53" s="69" t="n">
-        <v>14.09889328274008</v>
-      </c>
-      <c r="H53" s="23" t="n">
-        <v>15.38779817471642</v>
-      </c>
-      <c r="I53" s="69" t="n">
-        <v>14.45912210894593</v>
+        <v>16.51408925132097</v>
+      </c>
+      <c r="G53" s="68" t="n">
+        <v>14.09889440523192</v>
+      </c>
+      <c r="H53" s="21" t="n">
+        <v>15.38779834224254</v>
+      </c>
+      <c r="I53" s="68" t="n">
+        <v>14.45912441036983</v>
       </c>
       <c r="J53" s="5" t="n">
-        <v>17.48169294744561</v>
-      </c>
-      <c r="K53" s="21" t="n">
-        <v>25.61111509633099</v>
-      </c>
-      <c r="L53" s="21" t="n">
-        <v>23.62973982051687</v>
-      </c>
-      <c r="M53" s="69" t="n">
-        <v>59.46553030216641</v>
+        <v>17.48169356471491</v>
+      </c>
+      <c r="K53" s="61" t="n">
+        <v>25.61112164285462</v>
+      </c>
+      <c r="L53" s="61" t="n">
+        <v>23.62974030360016</v>
+      </c>
+      <c r="M53" s="68" t="n">
+        <v>59.465525699053</v>
       </c>
       <c r="N53" s="7" t="inlineStr"/>
     </row>
@@ -3484,7 +3484,7 @@
       <c r="A54" s="1" t="n">
         <v>52</v>
       </c>
-      <c r="B54" s="57" t="inlineStr">
+      <c r="B54" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3500,26 +3500,26 @@
         </is>
       </c>
       <c r="E54" s="3" t="inlineStr"/>
-      <c r="F54" s="21" t="n">
-        <v>17.18630050662639</v>
-      </c>
-      <c r="G54" s="64" t="n">
-        <v>45.40564447589527</v>
-      </c>
-      <c r="H54" s="71" t="n">
-        <v>30.20310548954298</v>
-      </c>
-      <c r="I54" s="73" t="n">
-        <v>16.32617580237585</v>
+      <c r="F54" s="61" t="n">
+        <v>17.18630064408944</v>
+      </c>
+      <c r="G54" s="63" t="n">
+        <v>45.40564448085657</v>
+      </c>
+      <c r="H54" s="70" t="n">
+        <v>30.20310106077959</v>
+      </c>
+      <c r="I54" s="72" t="n">
+        <v>16.32617764107752</v>
       </c>
       <c r="J54" s="5" t="n">
-        <v>17.47329781941077</v>
-      </c>
-      <c r="K54" s="73" t="n">
-        <v>20.21799422203556</v>
-      </c>
-      <c r="L54" s="21" t="n">
-        <v>25.14678852589688</v>
+        <v>17.47329790835571</v>
+      </c>
+      <c r="K54" s="72" t="n">
+        <v>20.21799626463999</v>
+      </c>
+      <c r="L54" s="61" t="n">
+        <v>25.14678858162365</v>
       </c>
       <c r="M54" s="7" t="inlineStr"/>
       <c r="N54" s="7" t="inlineStr"/>
@@ -3528,7 +3528,7 @@
       <c r="A55" s="1" t="n">
         <v>53</v>
       </c>
-      <c r="B55" s="57" t="inlineStr">
+      <c r="B55" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3544,29 +3544,29 @@
         </is>
       </c>
       <c r="E55" s="3" t="inlineStr"/>
-      <c r="F55" s="21" t="n">
-        <v>17.53516236275578</v>
-      </c>
-      <c r="G55" s="59" t="n">
-        <v>27.2278501332952</v>
-      </c>
-      <c r="H55" s="75" t="n">
-        <v>40.62378074457168</v>
+      <c r="F55" s="61" t="n">
+        <v>17.53516344013862</v>
+      </c>
+      <c r="G55" s="57" t="n">
+        <v>27.22785082993623</v>
+      </c>
+      <c r="H55" s="74" t="n">
+        <v>40.6237809051713</v>
       </c>
       <c r="I55" s="13" t="n">
-        <v>24.1832774752634</v>
-      </c>
-      <c r="J55" s="61" t="n">
-        <v>9.010619306482448</v>
+        <v>24.18327989748011</v>
+      </c>
+      <c r="J55" s="59" t="n">
+        <v>9.010619820308778</v>
       </c>
       <c r="K55" s="5" t="n">
-        <v>23.32516277792067</v>
-      </c>
-      <c r="L55" s="62" t="n">
-        <v>13.79390109864977</v>
+        <v>23.32516429287072</v>
+      </c>
+      <c r="L55" s="60" t="n">
+        <v>13.79390237890346</v>
       </c>
       <c r="M55" s="5" t="n">
-        <v>75.79566326846319</v>
+        <v>75.79565070842749</v>
       </c>
       <c r="N55" s="7" t="inlineStr"/>
     </row>
@@ -3574,7 +3574,7 @@
       <c r="A56" s="1" t="n">
         <v>54</v>
       </c>
-      <c r="B56" s="57" t="inlineStr">
+      <c r="B56" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3590,26 +3590,26 @@
         </is>
       </c>
       <c r="E56" s="3" t="inlineStr"/>
-      <c r="F56" s="71" t="n">
-        <v>21.29916546272529</v>
-      </c>
-      <c r="G56" s="76" t="n">
-        <v>94.36747574301634</v>
-      </c>
-      <c r="H56" s="67" t="n">
-        <v>56.34635126657046</v>
+      <c r="F56" s="70" t="n">
+        <v>21.29916728690715</v>
+      </c>
+      <c r="G56" s="75" t="n">
+        <v>94.36746004289701</v>
+      </c>
+      <c r="H56" s="66" t="n">
+        <v>56.34635625526007</v>
       </c>
       <c r="I56" s="16" t="n">
-        <v>21.29916546272529</v>
-      </c>
-      <c r="J56" s="62" t="n">
-        <v>10.29546760968708</v>
-      </c>
-      <c r="K56" s="71" t="n">
-        <v>30.41794380795807</v>
-      </c>
-      <c r="L56" s="65" t="n">
-        <v>68.28822694448731</v>
+        <v>21.29916728690715</v>
+      </c>
+      <c r="J56" s="60" t="n">
+        <v>10.29546823701846</v>
+      </c>
+      <c r="K56" s="70" t="n">
+        <v>30.4179439988874</v>
+      </c>
+      <c r="L56" s="64" t="n">
+        <v>68.2882210569754</v>
       </c>
       <c r="M56" s="7" t="inlineStr"/>
       <c r="N56" s="7" t="inlineStr"/>
@@ -3618,7 +3618,7 @@
       <c r="A57" s="1" t="n">
         <v>55</v>
       </c>
-      <c r="B57" s="57" t="inlineStr">
+      <c r="B57" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3634,29 +3634,29 @@
         </is>
       </c>
       <c r="E57" s="3" t="inlineStr"/>
-      <c r="F57" s="71" t="n">
-        <v>22.01316145501107</v>
-      </c>
-      <c r="G57" s="63" t="n">
-        <v>36.46815461087354</v>
+      <c r="F57" s="70" t="n">
+        <v>22.01316326832813</v>
+      </c>
+      <c r="G57" s="62" t="n">
+        <v>36.46815337329799</v>
       </c>
       <c r="H57" s="16" t="n">
-        <v>26.75370630485887</v>
+        <v>26.75370928357137</v>
       </c>
       <c r="I57" s="13" t="n">
-        <v>25.23889667872525</v>
-      </c>
-      <c r="J57" s="58" t="n">
-        <v>28.8139998816118</v>
+        <v>25.23889830736596</v>
+      </c>
+      <c r="J57" s="56" t="n">
+        <v>28.81399992309567</v>
       </c>
       <c r="K57" s="11" t="n">
-        <v>49.56382545567905</v>
-      </c>
-      <c r="L57" s="23" t="n">
-        <v>13.99645899470775</v>
-      </c>
-      <c r="M57" s="71" t="n">
-        <v>96.01878809640689</v>
+        <v>49.56382429803026</v>
+      </c>
+      <c r="L57" s="21" t="n">
+        <v>13.99645965882736</v>
+      </c>
+      <c r="M57" s="70" t="n">
+        <v>96.01877032401154</v>
       </c>
       <c r="N57" s="7" t="inlineStr"/>
     </row>
@@ -3664,7 +3664,7 @@
       <c r="A58" s="1" t="n">
         <v>56</v>
       </c>
-      <c r="B58" s="57" t="inlineStr">
+      <c r="B58" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3681,23 +3681,23 @@
       </c>
       <c r="E58" s="3" t="inlineStr"/>
       <c r="F58" s="13" t="n">
-        <v>22.35735287483737</v>
+        <v>22.27360714176167</v>
       </c>
       <c r="G58" s="16" t="n">
-        <v>22.28677227608177</v>
-      </c>
-      <c r="H58" s="71" t="n">
-        <v>29.38386530768343</v>
-      </c>
-      <c r="I58" s="71" t="n">
-        <v>23.5851456077105</v>
-      </c>
-      <c r="J58" s="68" t="n">
-        <v>31.8053036716978</v>
+        <v>22.05905699239992</v>
+      </c>
+      <c r="H58" s="70" t="n">
+        <v>29.38386429902256</v>
+      </c>
+      <c r="I58" s="70" t="n">
+        <v>23.58514582833682</v>
+      </c>
+      <c r="J58" s="67" t="n">
+        <v>31.8053059562663</v>
       </c>
       <c r="K58" s="7" t="inlineStr"/>
-      <c r="L58" s="61" t="n">
-        <v>9.570240471375332</v>
+      <c r="L58" s="59" t="n">
+        <v>9.570241102321955</v>
       </c>
       <c r="M58" s="7" t="inlineStr"/>
       <c r="N58" s="7" t="inlineStr"/>
@@ -3706,7 +3706,7 @@
       <c r="A59" s="1" t="n">
         <v>57</v>
       </c>
-      <c r="B59" s="57" t="inlineStr">
+      <c r="B59" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3723,25 +3723,25 @@
       </c>
       <c r="E59" s="3" t="inlineStr"/>
       <c r="F59" s="13" t="n">
-        <v>23.08857951886908</v>
-      </c>
-      <c r="G59" s="58" t="n">
-        <v>30.6334760845553</v>
-      </c>
-      <c r="H59" s="71" t="n">
-        <v>29.59420223438968</v>
-      </c>
-      <c r="I59" s="73" t="n">
-        <v>15.85774115666421</v>
-      </c>
-      <c r="J59" s="66" t="n">
-        <v>37.43045214342968</v>
-      </c>
-      <c r="K59" s="63" t="n">
-        <v>45.29351768763168</v>
-      </c>
-      <c r="L59" s="21" t="n">
-        <v>24.85197963182721</v>
+        <v>23.08858125522978</v>
+      </c>
+      <c r="G59" s="56" t="n">
+        <v>30.63347479162304</v>
+      </c>
+      <c r="H59" s="70" t="n">
+        <v>29.59420309451453</v>
+      </c>
+      <c r="I59" s="72" t="n">
+        <v>15.85774247896939</v>
+      </c>
+      <c r="J59" s="65" t="n">
+        <v>37.43045557938333</v>
+      </c>
+      <c r="K59" s="62" t="n">
+        <v>45.29351960605806</v>
+      </c>
+      <c r="L59" s="61" t="n">
+        <v>24.85198120044492</v>
       </c>
       <c r="M59" s="7" t="inlineStr"/>
       <c r="N59" s="7" t="inlineStr"/>
@@ -3750,7 +3750,7 @@
       <c r="A60" s="1" t="n">
         <v>58</v>
       </c>
-      <c r="B60" s="57" t="inlineStr">
+      <c r="B60" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3767,28 +3767,28 @@
       </c>
       <c r="E60" s="3" t="inlineStr"/>
       <c r="F60" s="19" t="n">
-        <v>38.92470647227253</v>
-      </c>
-      <c r="G60" s="25" t="n">
-        <v>70.75067956891191</v>
-      </c>
-      <c r="H60" s="66" t="n">
-        <v>44.9436136443224</v>
-      </c>
-      <c r="I60" s="77" t="n">
-        <v>61.6315875200706</v>
+        <v>38.92470642836854</v>
+      </c>
+      <c r="G60" s="24" t="n">
+        <v>70.75067881568536</v>
+      </c>
+      <c r="H60" s="65" t="n">
+        <v>44.94361522969408</v>
+      </c>
+      <c r="I60" s="76" t="n">
+        <v>61.63158358184176</v>
       </c>
       <c r="J60" s="13" t="n">
-        <v>25.4923506144501</v>
-      </c>
-      <c r="K60" s="78" t="n">
-        <v>60.83033414542964</v>
-      </c>
-      <c r="L60" s="30" t="n">
-        <v>97.9206391891485</v>
-      </c>
-      <c r="M60" s="71" t="n">
-        <v>94.97594944702669</v>
+        <v>25.49235112400903</v>
+      </c>
+      <c r="K60" s="77" t="n">
+        <v>60.83033473397547</v>
+      </c>
+      <c r="L60" s="78" t="n">
+        <v>97.92062383003802</v>
+      </c>
+      <c r="M60" s="70" t="n">
+        <v>94.97593273367737</v>
       </c>
       <c r="N60" s="7" t="inlineStr"/>
     </row>
@@ -3796,7 +3796,7 @@
       <c r="A61" s="1" t="n">
         <v>59</v>
       </c>
-      <c r="B61" s="57" t="inlineStr">
+      <c r="B61" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3811,7 +3811,7 @@
           <t>Palmitamide</t>
         </is>
       </c>
-      <c r="E61" s="56" t="inlineStr">
+      <c r="E61" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -3830,7 +3830,7 @@
       <c r="A62" s="1" t="n">
         <v>60</v>
       </c>
-      <c r="B62" s="57" t="inlineStr">
+      <c r="B62" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3845,7 +3845,7 @@
           <t>p-Coumaric acid</t>
         </is>
       </c>
-      <c r="E62" s="56" t="inlineStr">
+      <c r="E62" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -3864,7 +3864,7 @@
       <c r="A63" s="1" t="n">
         <v>61</v>
       </c>
-      <c r="B63" s="57" t="inlineStr">
+      <c r="B63" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3879,7 +3879,7 @@
           <t>Theophylline</t>
         </is>
       </c>
-      <c r="E63" s="56" t="inlineStr">
+      <c r="E63" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -3898,7 +3898,7 @@
       <c r="A64" s="1" t="n">
         <v>62</v>
       </c>
-      <c r="B64" s="57" t="inlineStr">
+      <c r="B64" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3913,7 +3913,7 @@
           <t>Theobromine</t>
         </is>
       </c>
-      <c r="E64" s="56" t="inlineStr">
+      <c r="E64" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -3932,7 +3932,7 @@
       <c r="A65" s="1" t="n">
         <v>63</v>
       </c>
-      <c r="B65" s="57" t="inlineStr">
+      <c r="B65" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3947,7 +3947,7 @@
           <t>Withanoside V</t>
         </is>
       </c>
-      <c r="E65" s="56" t="inlineStr">
+      <c r="E65" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -3966,7 +3966,7 @@
       <c r="A66" s="1" t="n">
         <v>64</v>
       </c>
-      <c r="B66" s="57" t="inlineStr">
+      <c r="B66" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -3981,7 +3981,7 @@
           <t>(-)-Catechin</t>
         </is>
       </c>
-      <c r="E66" s="56" t="inlineStr">
+      <c r="E66" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4000,7 +4000,7 @@
       <c r="A67" s="1" t="n">
         <v>65</v>
       </c>
-      <c r="B67" s="57" t="inlineStr">
+      <c r="B67" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4015,7 +4015,7 @@
           <t>7-Acetylintermedine N-oxide</t>
         </is>
       </c>
-      <c r="E67" s="56" t="inlineStr">
+      <c r="E67" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4034,7 +4034,7 @@
       <c r="A68" s="1" t="n">
         <v>66</v>
       </c>
-      <c r="B68" s="57" t="inlineStr">
+      <c r="B68" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4049,7 +4049,7 @@
           <t>Ginsenoside Rb3</t>
         </is>
       </c>
-      <c r="E68" s="56" t="inlineStr">
+      <c r="E68" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4068,7 +4068,7 @@
       <c r="A69" s="1" t="n">
         <v>67</v>
       </c>
-      <c r="B69" s="57" t="inlineStr">
+      <c r="B69" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4083,7 +4083,7 @@
           <t>Withanoside IV</t>
         </is>
       </c>
-      <c r="E69" s="56" t="inlineStr">
+      <c r="E69" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4095,8 +4095,8 @@
       <c r="J69" s="7" t="inlineStr"/>
       <c r="K69" s="7" t="inlineStr"/>
       <c r="L69" s="7" t="inlineStr"/>
-      <c r="M69" s="71" t="n">
-        <v>99.68867822053444</v>
+      <c r="M69" s="70" t="n">
+        <v>99.68865811814057</v>
       </c>
       <c r="N69" s="7" t="inlineStr"/>
     </row>
@@ -4104,7 +4104,7 @@
       <c r="A70" s="1" t="n">
         <v>68</v>
       </c>
-      <c r="B70" s="57" t="inlineStr">
+      <c r="B70" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4119,7 +4119,7 @@
           <t>Ginsenoside Rg1</t>
         </is>
       </c>
-      <c r="E70" s="56" t="inlineStr">
+      <c r="E70" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4138,7 +4138,7 @@
       <c r="A71" s="1" t="n">
         <v>69</v>
       </c>
-      <c r="B71" s="57" t="inlineStr">
+      <c r="B71" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4153,7 +4153,7 @@
           <t>Lycopsamine-N-oxide</t>
         </is>
       </c>
-      <c r="E71" s="56" t="inlineStr">
+      <c r="E71" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4172,7 +4172,7 @@
       <c r="A72" s="1" t="n">
         <v>70</v>
       </c>
-      <c r="B72" s="57" t="inlineStr">
+      <c r="B72" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4187,7 +4187,7 @@
           <t>Ginsenoside Re</t>
         </is>
       </c>
-      <c r="E72" s="56" t="inlineStr">
+      <c r="E72" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4199,8 +4199,8 @@
       <c r="J72" s="7" t="inlineStr"/>
       <c r="K72" s="7" t="inlineStr"/>
       <c r="L72" s="7" t="inlineStr"/>
-      <c r="M72" s="21" t="n">
-        <v>82.84540659738045</v>
+      <c r="M72" s="61" t="n">
+        <v>82.84538548111971</v>
       </c>
       <c r="N72" s="7" t="inlineStr"/>
     </row>
@@ -4208,7 +4208,7 @@
       <c r="A73" s="1" t="n">
         <v>71</v>
       </c>
-      <c r="B73" s="57" t="inlineStr">
+      <c r="B73" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4223,7 +4223,7 @@
           <t>7-Acetyllycopsamine</t>
         </is>
       </c>
-      <c r="E73" s="56" t="inlineStr">
+      <c r="E73" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4242,7 +4242,7 @@
       <c r="A74" s="1" t="n">
         <v>72</v>
       </c>
-      <c r="B74" s="57" t="inlineStr">
+      <c r="B74" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4257,7 +4257,7 @@
           <t>Magnoflorine</t>
         </is>
       </c>
-      <c r="E74" s="56" t="inlineStr">
+      <c r="E74" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4276,7 +4276,7 @@
       <c r="A75" s="1" t="n">
         <v>73</v>
       </c>
-      <c r="B75" s="57" t="inlineStr">
+      <c r="B75" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4291,7 +4291,7 @@
           <t>Ginsenoside Rb1</t>
         </is>
       </c>
-      <c r="E75" s="56" t="inlineStr">
+      <c r="E75" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4303,8 +4303,8 @@
       <c r="J75" s="7" t="inlineStr"/>
       <c r="K75" s="7" t="inlineStr"/>
       <c r="L75" s="7" t="inlineStr"/>
-      <c r="M75" s="62" t="n">
-        <v>42.99254294786281</v>
+      <c r="M75" s="60" t="n">
+        <v>42.99254342208955</v>
       </c>
       <c r="N75" s="7" t="inlineStr"/>
     </row>
@@ -4312,7 +4312,7 @@
       <c r="A76" s="1" t="n">
         <v>74</v>
       </c>
-      <c r="B76" s="57" t="inlineStr">
+      <c r="B76" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4327,7 +4327,7 @@
           <t>Lycopsamine</t>
         </is>
       </c>
-      <c r="E76" s="56" t="inlineStr">
+      <c r="E76" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4339,8 +4339,8 @@
       <c r="J76" s="7" t="inlineStr"/>
       <c r="K76" s="7" t="inlineStr"/>
       <c r="L76" s="7" t="inlineStr"/>
-      <c r="M76" s="61" t="n">
-        <v>38.13363910920266</v>
+      <c r="M76" s="59" t="n">
+        <v>38.13363663722031</v>
       </c>
       <c r="N76" s="7" t="inlineStr"/>
     </row>
@@ -4348,7 +4348,7 @@
       <c r="A77" s="1" t="n">
         <v>75</v>
       </c>
-      <c r="B77" s="57" t="inlineStr">
+      <c r="B77" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4363,7 +4363,7 @@
           <t>7-Acetyllycopsamine N-oxide</t>
         </is>
       </c>
-      <c r="E77" s="56" t="inlineStr">
+      <c r="E77" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4382,7 +4382,7 @@
       <c r="A78" s="1" t="n">
         <v>76</v>
       </c>
-      <c r="B78" s="57" t="inlineStr">
+      <c r="B78" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4397,7 +4397,7 @@
           <t>Ginsenoside Rb2</t>
         </is>
       </c>
-      <c r="E78" s="56" t="inlineStr">
+      <c r="E78" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4416,7 +4416,7 @@
       <c r="A79" s="1" t="n">
         <v>77</v>
       </c>
-      <c r="B79" s="57" t="inlineStr">
+      <c r="B79" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4431,7 +4431,7 @@
           <t>(−)-Epigallocatechin-3-O-gallate</t>
         </is>
       </c>
-      <c r="E79" s="56" t="inlineStr">
+      <c r="E79" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4443,8 +4443,8 @@
       <c r="J79" s="7" t="inlineStr"/>
       <c r="K79" s="7" t="inlineStr"/>
       <c r="L79" s="7" t="inlineStr"/>
-      <c r="M79" s="73" t="n">
-        <v>66.33294026887933</v>
+      <c r="M79" s="72" t="n">
+        <v>66.33294053770604</v>
       </c>
       <c r="N79" s="7" t="inlineStr"/>
     </row>
@@ -4452,7 +4452,7 @@
       <c r="A80" s="1" t="n">
         <v>78</v>
       </c>
-      <c r="B80" s="57" t="inlineStr">
+      <c r="B80" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4467,7 +4467,7 @@
           <t>(D)-Catechin</t>
         </is>
       </c>
-      <c r="E80" s="56" t="inlineStr">
+      <c r="E80" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4486,7 +4486,7 @@
       <c r="A81" s="1" t="n">
         <v>79</v>
       </c>
-      <c r="B81" s="57" t="inlineStr">
+      <c r="B81" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4501,7 +4501,7 @@
           <t>trans-Chlorogenic acid</t>
         </is>
       </c>
-      <c r="E81" s="56" t="inlineStr">
+      <c r="E81" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4513,8 +4513,8 @@
       <c r="J81" s="7" t="inlineStr"/>
       <c r="K81" s="7" t="inlineStr"/>
       <c r="L81" s="7" t="inlineStr"/>
-      <c r="M81" s="71" t="n">
-        <v>98.79727367587026</v>
+      <c r="M81" s="70" t="n">
+        <v>98.79725742261499</v>
       </c>
       <c r="N81" s="7" t="inlineStr"/>
     </row>
@@ -4522,7 +4522,7 @@
       <c r="A82" s="1" t="n">
         <v>80</v>
       </c>
-      <c r="B82" s="57" t="inlineStr">
+      <c r="B82" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4537,7 +4537,7 @@
           <t>Epicatechin</t>
         </is>
       </c>
-      <c r="E82" s="56" t="inlineStr">
+      <c r="E82" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4550,15 +4550,15 @@
       <c r="K82" s="7" t="inlineStr"/>
       <c r="L82" s="7" t="inlineStr"/>
       <c r="M82" s="7" t="inlineStr"/>
-      <c r="N82" s="74" t="n">
-        <v>56.68135763132471</v>
+      <c r="N82" s="73" t="n">
+        <v>56.68135138467033</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="1" t="n">
         <v>81</v>
       </c>
-      <c r="B83" s="57" t="inlineStr">
+      <c r="B83" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4573,7 +4573,7 @@
           <t>Caffeine</t>
         </is>
       </c>
-      <c r="E83" s="56" t="inlineStr">
+      <c r="E83" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4592,7 +4592,7 @@
       <c r="A84" s="1" t="n">
         <v>82</v>
       </c>
-      <c r="B84" s="57" t="inlineStr">
+      <c r="B84" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4607,7 +4607,7 @@
           <t>Taxifolin</t>
         </is>
       </c>
-      <c r="E84" s="56" t="inlineStr">
+      <c r="E84" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4626,7 +4626,7 @@
       <c r="A85" s="1" t="n">
         <v>83</v>
       </c>
-      <c r="B85" s="57" t="inlineStr">
+      <c r="B85" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4641,7 +4641,7 @@
           <t>(−)-Epigallocatechin</t>
         </is>
       </c>
-      <c r="E85" s="56" t="inlineStr">
+      <c r="E85" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4660,7 +4660,7 @@
       <c r="A86" s="1" t="n">
         <v>84</v>
       </c>
-      <c r="B86" s="57" t="inlineStr">
+      <c r="B86" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4675,7 +4675,7 @@
           <t>Gallic acid</t>
         </is>
       </c>
-      <c r="E86" s="56" t="inlineStr">
+      <c r="E86" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4687,8 +4687,8 @@
       <c r="J86" s="7" t="inlineStr"/>
       <c r="K86" s="7" t="inlineStr"/>
       <c r="L86" s="7" t="inlineStr"/>
-      <c r="M86" s="23" t="n">
-        <v>50.75524528300282</v>
+      <c r="M86" s="21" t="n">
+        <v>50.75524435566008</v>
       </c>
       <c r="N86" s="7" t="inlineStr"/>
     </row>
@@ -4696,7 +4696,7 @@
       <c r="A87" s="1" t="n">
         <v>85</v>
       </c>
-      <c r="B87" s="57" t="inlineStr">
+      <c r="B87" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4711,7 +4711,7 @@
           <t>7,8-Dihydrokavain</t>
         </is>
       </c>
-      <c r="E87" s="56" t="inlineStr">
+      <c r="E87" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4730,7 +4730,7 @@
       <c r="A88" s="1" t="n">
         <v>86</v>
       </c>
-      <c r="B88" s="57" t="inlineStr">
+      <c r="B88" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4745,7 +4745,7 @@
           <t>Yohimbic acid</t>
         </is>
       </c>
-      <c r="E88" s="56" t="inlineStr">
+      <c r="E88" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4757,8 +4757,8 @@
       <c r="J88" s="7" t="inlineStr"/>
       <c r="K88" s="7" t="inlineStr"/>
       <c r="L88" s="7" t="inlineStr"/>
-      <c r="M88" s="21" t="n">
-        <v>81.13799789362174</v>
+      <c r="M88" s="61" t="n">
+        <v>81.13798390318806</v>
       </c>
       <c r="N88" s="7" t="inlineStr"/>
     </row>
@@ -4766,7 +4766,7 @@
       <c r="A89" s="1" t="n">
         <v>87</v>
       </c>
-      <c r="B89" s="57" t="inlineStr">
+      <c r="B89" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4781,7 +4781,7 @@
           <t>Withanolide B</t>
         </is>
       </c>
-      <c r="E89" s="56" t="inlineStr">
+      <c r="E89" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4793,8 +4793,8 @@
       <c r="J89" s="7" t="inlineStr"/>
       <c r="K89" s="7" t="inlineStr"/>
       <c r="L89" s="7" t="inlineStr"/>
-      <c r="M89" s="23" t="n">
-        <v>49.3697695457037</v>
+      <c r="M89" s="21" t="n">
+        <v>49.36977307824154</v>
       </c>
       <c r="N89" s="7" t="inlineStr"/>
     </row>
@@ -4802,7 +4802,7 @@
       <c r="A90" s="1" t="n">
         <v>88</v>
       </c>
-      <c r="B90" s="57" t="inlineStr">
+      <c r="B90" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4817,7 +4817,7 @@
           <t>Lupanine</t>
         </is>
       </c>
-      <c r="E90" s="56" t="inlineStr">
+      <c r="E90" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4836,7 +4836,7 @@
       <c r="A91" s="1" t="n">
         <v>89</v>
       </c>
-      <c r="B91" s="57" t="inlineStr">
+      <c r="B91" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4851,7 +4851,7 @@
           <t>Ginsenoside Ra2</t>
         </is>
       </c>
-      <c r="E91" s="56" t="inlineStr">
+      <c r="E91" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4870,7 +4870,7 @@
       <c r="A92" s="1" t="n">
         <v>90</v>
       </c>
-      <c r="B92" s="57" t="inlineStr">
+      <c r="B92" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4885,7 +4885,7 @@
           <t>N-methylcytisine</t>
         </is>
       </c>
-      <c r="E92" s="56" t="inlineStr">
+      <c r="E92" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4904,7 +4904,7 @@
       <c r="A93" s="1" t="n">
         <v>91</v>
       </c>
-      <c r="B93" s="57" t="inlineStr">
+      <c r="B93" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4919,7 +4919,7 @@
           <t>Kavain</t>
         </is>
       </c>
-      <c r="E93" s="56" t="inlineStr">
+      <c r="E93" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4938,7 +4938,7 @@
       <c r="A94" s="1" t="n">
         <v>92</v>
       </c>
-      <c r="B94" s="57" t="inlineStr">
+      <c r="B94" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4953,7 +4953,7 @@
           <t>Notoginsenoside R2</t>
         </is>
       </c>
-      <c r="E94" s="56" t="inlineStr">
+      <c r="E94" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -4972,7 +4972,7 @@
       <c r="A95" s="1" t="n">
         <v>93</v>
       </c>
-      <c r="B95" s="57" t="inlineStr">
+      <c r="B95" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -4987,7 +4987,7 @@
           <t>Acetylglutamic acid</t>
         </is>
       </c>
-      <c r="E95" s="56" t="inlineStr">
+      <c r="E95" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -5006,7 +5006,7 @@
       <c r="A96" s="1" t="n">
         <v>94</v>
       </c>
-      <c r="B96" s="57" t="inlineStr">
+      <c r="B96" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -5021,7 +5021,7 @@
           <t>Pyroglutamic acid</t>
         </is>
       </c>
-      <c r="E96" s="56" t="inlineStr">
+      <c r="E96" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -5034,7 +5034,7 @@
       <c r="K96" s="7" t="inlineStr"/>
       <c r="L96" s="7" t="inlineStr"/>
       <c r="M96" s="4" t="n">
-        <v>6.534473316406666</v>
+        <v>6.534474197154031</v>
       </c>
       <c r="N96" s="7" t="inlineStr"/>
     </row>
@@ -5042,7 +5042,7 @@
       <c r="A97" s="1" t="n">
         <v>95</v>
       </c>
-      <c r="B97" s="57" t="inlineStr">
+      <c r="B97" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -5057,7 +5057,7 @@
           <t>Methylsticin</t>
         </is>
       </c>
-      <c r="E97" s="56" t="inlineStr">
+      <c r="E97" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>
@@ -5076,7 +5076,7 @@
       <c r="A98" s="1" t="n">
         <v>96</v>
       </c>
-      <c r="B98" s="57" t="inlineStr">
+      <c r="B98" s="55" t="inlineStr">
         <is>
           <t>Constituent</t>
         </is>
@@ -5091,7 +5091,7 @@
           <t>Baptifoline</t>
         </is>
       </c>
-      <c r="E98" s="56" t="inlineStr">
+      <c r="E98" s="54" t="inlineStr">
         <is>
           <t>✗</t>
         </is>

</xml_diff>